<commit_message>
cleaned up folders, all data central to DATA folder, created viz folder
</commit_message>
<xml_diff>
--- a/DATA/ARCHIVE/production_capacity_updated.xlsx
+++ b/DATA/ARCHIVE/production_capacity_updated.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27531"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5e6b18ad1acc1266/Desktop/Vaccine_Tender/horizon excursion/50 years/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5e6b18ad1acc1266/Desktop/Vaccine_Tender/DATA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="200" documentId="13_ncr:1_{68782C53-48E3-42CA-912A-5E0671CC39DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6729F7D9-DC3C-4C02-98A0-5B34E1980364}"/>
+  <xr:revisionPtr revIDLastSave="75" documentId="13_ncr:1_{5BC75AC5-5DFF-42F9-8F6A-B58AA24898A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C2477377-9AD5-4BDA-B66E-AB3748EB6E49}"/>
   <bookViews>
-    <workbookView xWindow="13550" yWindow="-110" windowWidth="38620" windowHeight="21100" firstSheet="1" activeTab="4" xr2:uid="{752E71BE-3FD4-4CCA-ABF0-6C5710D300B4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{752E71BE-3FD4-4CCA-ABF0-6C5710D300B4}"/>
   </bookViews>
   <sheets>
     <sheet name="vaccine-producer list" sheetId="8" r:id="rId1"/>
@@ -18,10 +18,9 @@
     <sheet name="Prod_capacity_agg" sheetId="9" r:id="rId3"/>
     <sheet name="Producers_short_name" sheetId="5" r:id="rId4"/>
     <sheet name="Medium_Capacity" sheetId="6" r:id="rId5"/>
-    <sheet name="Sheet1" sheetId="10" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Medium_Capacity!$A$2:$O$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Medium_Capacity!$A$1:$K$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Prod_capacity_agg!$A$1:$K$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">total_capacity_calcs!$A$229:$L$296</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'vaccine-producer list'!$A$1:$R$54</definedName>
@@ -31,7 +30,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId7"/>
+    <pivotCache cacheId="0" r:id="rId6"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -189,7 +188,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="757" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="757" uniqueCount="171">
   <si>
     <t>Vaccine</t>
   </si>
@@ -671,6 +670,9 @@
     <t>"Pfizer"</t>
   </si>
   <si>
+    <t>"Innovative_Biotech"</t>
+  </si>
+  <si>
     <t>Sum of 1</t>
   </si>
   <si>
@@ -699,12 +701,6 @@
   </si>
   <si>
     <t>Sum of 10</t>
-  </si>
-  <si>
-    <t>Producer X</t>
-  </si>
-  <si>
-    <t>"Producer_X"</t>
   </si>
 </sst>
 </file>
@@ -1020,8 +1016,10 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="4" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2387,7 +2385,7 @@
         <v>156</v>
       </c>
       <c r="T1" s="33" t="s">
-        <v>170</v>
+        <v>154</v>
       </c>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.25">
@@ -10278,11 +10276,11 @@
         <v>110</v>
       </c>
       <c r="C207" s="8">
-        <f t="shared" ref="C207:L207" si="0">SUM(C96+C136+C142)</f>
-        <v>14777182.228013158</v>
+        <f>SUM(C96+C136+C132)</f>
+        <v>12398505.803013157</v>
       </c>
       <c r="D207" s="8">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="C207:L207" si="0">SUM(D96+D136+D142)</f>
         <v>37949221.241086259</v>
       </c>
       <c r="E207" s="8">
@@ -11126,7 +11124,7 @@
       <c r="K228" s="15"/>
       <c r="L228" s="15"/>
     </row>
-    <row r="229" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B229" s="2" t="s">
         <v>115</v>
       </c>
@@ -11136,13 +11134,13 @@
       <c r="K229" s="27"/>
       <c r="L229" s="27"/>
     </row>
-    <row r="230" spans="1:12" s="19" customFormat="1" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:12" s="19" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A230" s="18" t="s">
         <v>43</v>
       </c>
       <c r="C230" s="19">
         <f t="shared" ref="C230:L230" si="17">C207*$B226</f>
-        <v>13299464.005211843</v>
+        <v>11158655.222711843</v>
       </c>
       <c r="D230" s="19">
         <f t="shared" si="17"/>
@@ -11190,7 +11188,7 @@
       </c>
       <c r="C231" s="2">
         <f t="shared" ref="C231:L231" si="18">$B$231*C230</f>
-        <v>10881379.640627872</v>
+        <v>9129808.8185824174</v>
       </c>
       <c r="D231" s="2">
         <f t="shared" si="18"/>
@@ -11229,7 +11227,7 @@
         <v>16872659.841640912</v>
       </c>
     </row>
-    <row r="232" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A232" s="2" t="s">
         <v>118</v>
       </c>
@@ -11238,7 +11236,7 @@
       </c>
       <c r="C232" s="2">
         <f t="shared" ref="C232:L232" si="19">$B$232*C230</f>
-        <v>2418084.364583971</v>
+        <v>2028846.4041294253</v>
       </c>
       <c r="D232" s="2">
         <f t="shared" si="19"/>
@@ -11277,7 +11275,7 @@
         <v>3749479.9648090904</v>
       </c>
     </row>
-    <row r="233" spans="1:12" s="19" customFormat="1" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:12" s="19" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A233" s="18" t="s">
         <v>57</v>
       </c>
@@ -14471,34 +14469,34 @@
         <v>121</v>
       </c>
       <c r="N3" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="O3" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="P3" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="Q3" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="R3" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="S3" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T3" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="U3" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="V3" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="W3" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="4" spans="1:23" x14ac:dyDescent="0.25">
@@ -15901,34 +15899,34 @@
         <v>121</v>
       </c>
       <c r="N25" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="O25" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="P25" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="Q25" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="R25" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="S25" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="T25" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="U25" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="V25" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="W25" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.25">
@@ -18309,7 +18307,6 @@
   <cols>
     <col min="2" max="2" width="39.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="25.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="217.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:20" x14ac:dyDescent="0.25">
@@ -18566,10 +18563,10 @@
     </row>
     <row r="19" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B19" s="26" t="s">
-        <v>170</v>
+        <v>154</v>
       </c>
       <c r="C19" s="26" t="s">
-        <v>171</v>
+        <v>160</v>
       </c>
     </row>
   </sheetData>
@@ -18580,20 +18577,14 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DF17EB8-02F1-485E-9D81-51CF2F0BE0EA}">
-  <dimension ref="A1:AY44"/>
+  <dimension ref="A1:K44"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="11" width="12.7109375" customWidth="1"/>
-    <col min="12" max="12" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="11" width="14.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B1" s="36">
         <v>1</v>
       </c>
@@ -18624,3443 +18615,603 @@
       <c r="K1" s="36">
         <v>10</v>
       </c>
-      <c r="L1" s="36">
-        <v>11</v>
-      </c>
-      <c r="M1" s="36">
-        <v>12</v>
-      </c>
-      <c r="N1" s="36">
-        <v>13</v>
-      </c>
-      <c r="O1" s="36">
-        <v>14</v>
-      </c>
-      <c r="P1" s="36">
-        <v>15</v>
-      </c>
-      <c r="Q1" s="36">
-        <v>16</v>
-      </c>
-      <c r="R1" s="36">
-        <v>17</v>
-      </c>
-      <c r="S1" s="36">
-        <v>18</v>
-      </c>
-      <c r="T1" s="36">
-        <v>19</v>
-      </c>
-      <c r="U1" s="36">
-        <v>20</v>
-      </c>
-      <c r="V1" s="36">
-        <v>21</v>
-      </c>
-      <c r="W1" s="36">
-        <v>22</v>
-      </c>
-      <c r="X1" s="36">
-        <v>23</v>
-      </c>
-      <c r="Y1" s="36">
-        <v>24</v>
-      </c>
-      <c r="Z1" s="36">
-        <v>25</v>
-      </c>
-      <c r="AA1" s="36">
-        <v>26</v>
-      </c>
-      <c r="AB1" s="36">
-        <v>27</v>
-      </c>
-      <c r="AC1" s="36">
-        <v>28</v>
-      </c>
-      <c r="AD1" s="36">
-        <v>29</v>
-      </c>
-      <c r="AE1" s="36">
-        <v>30</v>
-      </c>
-      <c r="AF1" s="36">
-        <v>31</v>
-      </c>
-      <c r="AG1" s="36">
-        <v>32</v>
-      </c>
-      <c r="AH1" s="36">
-        <v>33</v>
-      </c>
-      <c r="AI1" s="36">
-        <v>34</v>
-      </c>
-      <c r="AJ1" s="36">
-        <v>35</v>
-      </c>
-      <c r="AK1" s="36">
-        <v>36</v>
-      </c>
-      <c r="AL1" s="36">
-        <v>37</v>
-      </c>
-      <c r="AM1" s="36">
-        <v>38</v>
-      </c>
-      <c r="AN1" s="36">
-        <v>39</v>
-      </c>
-      <c r="AO1" s="36">
-        <v>40</v>
-      </c>
-      <c r="AP1" s="36">
-        <v>41</v>
-      </c>
-      <c r="AQ1" s="36">
-        <v>42</v>
-      </c>
-      <c r="AR1" s="36">
-        <v>43</v>
-      </c>
-      <c r="AS1" s="36">
-        <v>44</v>
-      </c>
-      <c r="AT1" s="36">
-        <v>45</v>
-      </c>
-      <c r="AU1" s="36">
-        <v>46</v>
-      </c>
-      <c r="AV1" s="36">
-        <v>47</v>
-      </c>
-      <c r="AW1" s="36">
-        <v>48</v>
-      </c>
-      <c r="AX1" s="36">
-        <v>49</v>
-      </c>
-      <c r="AY1" s="36">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="2" spans="1:51" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B2" s="37">
+        <v>1733000000</v>
+      </c>
+      <c r="C2" s="37">
+        <v>1921000000</v>
+      </c>
+      <c r="D2" s="37">
+        <v>2079000000</v>
+      </c>
+      <c r="E2" s="37">
+        <v>2391000000</v>
+      </c>
+      <c r="F2" s="37">
+        <v>2603000000</v>
+      </c>
+      <c r="G2" s="37">
+        <v>2371000000</v>
+      </c>
+      <c r="H2" s="37">
+        <v>2251000000</v>
+      </c>
+      <c r="I2" s="37">
+        <v>2198000000</v>
+      </c>
+      <c r="J2" s="37">
+        <v>2155000000</v>
+      </c>
+      <c r="K2" s="37">
+        <v>2178000000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>144</v>
+      </c>
+      <c r="B3" s="37">
+        <v>160100000</v>
+      </c>
+      <c r="C3" s="37">
+        <v>140800000</v>
+      </c>
+      <c r="D3" s="37">
+        <v>154800000</v>
+      </c>
+      <c r="E3" s="37">
+        <v>143800000</v>
+      </c>
+      <c r="F3" s="37">
+        <v>147500000</v>
+      </c>
+      <c r="G3" s="37">
+        <v>171200000</v>
+      </c>
+      <c r="H3" s="37">
+        <v>139700000</v>
+      </c>
+      <c r="I3" s="37">
+        <v>172900000</v>
+      </c>
+      <c r="J3" s="37">
+        <v>149300000</v>
+      </c>
+      <c r="K3" s="37">
+        <v>158400000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>148</v>
+      </c>
+      <c r="B4" s="37">
+        <v>248000000</v>
+      </c>
+      <c r="C4" s="37">
+        <v>248000000</v>
+      </c>
+      <c r="D4" s="37">
+        <v>360000000</v>
+      </c>
+      <c r="E4" s="37">
+        <v>952000000</v>
+      </c>
+      <c r="F4" s="37">
+        <v>1216000000</v>
+      </c>
+      <c r="G4" s="37">
+        <v>848000000</v>
+      </c>
+      <c r="H4" s="37">
+        <v>552000000</v>
+      </c>
+      <c r="I4" s="37">
+        <v>552000000</v>
+      </c>
+      <c r="J4" s="37">
+        <v>440000000</v>
+      </c>
+      <c r="K4" s="37">
+        <v>456000000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>150</v>
+      </c>
+      <c r="B5" s="37">
+        <v>116600000</v>
+      </c>
+      <c r="C5" s="37">
+        <v>129900000</v>
+      </c>
+      <c r="D5" s="37">
+        <v>128200000</v>
+      </c>
+      <c r="E5" s="37">
+        <v>123000000</v>
+      </c>
+      <c r="F5" s="37">
+        <v>123100000</v>
+      </c>
+      <c r="G5" s="37">
+        <v>120400000</v>
+      </c>
+      <c r="H5" s="37">
+        <v>121900000</v>
+      </c>
+      <c r="I5" s="37">
+        <v>121000000</v>
+      </c>
+      <c r="J5" s="37">
+        <v>122400000</v>
+      </c>
+      <c r="K5" s="37">
+        <v>123300000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>152</v>
+      </c>
+      <c r="B6">
+        <v>1074100000</v>
+      </c>
+      <c r="C6">
+        <v>1109700000</v>
+      </c>
+      <c r="D6">
+        <v>1160000000</v>
+      </c>
+      <c r="E6">
+        <v>1115800000</v>
+      </c>
+      <c r="F6">
+        <v>1141600000</v>
+      </c>
+      <c r="G6">
+        <v>1191500000</v>
+      </c>
+      <c r="H6">
+        <v>1120400000</v>
+      </c>
+      <c r="I6">
+        <v>1192500000</v>
+      </c>
+      <c r="J6">
+        <v>1139200000</v>
+      </c>
+      <c r="K6">
+        <v>1169600000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>123</v>
       </c>
-      <c r="B2" s="37">
+      <c r="B7" s="37">
         <v>12600000</v>
       </c>
-      <c r="C2" s="37">
+      <c r="C7" s="37">
         <v>16800000</v>
       </c>
-      <c r="D2" s="37">
+      <c r="D7" s="37">
         <v>19600000</v>
       </c>
-      <c r="E2" s="37">
+      <c r="E7" s="37">
         <v>19500000</v>
       </c>
-      <c r="F2" s="37">
+      <c r="F7" s="37">
         <v>19500000</v>
       </c>
-      <c r="G2" s="37">
+      <c r="G7" s="37">
         <v>19200000</v>
       </c>
-      <c r="H2" s="37">
+      <c r="H7" s="37">
         <v>19600000</v>
       </c>
-      <c r="I2" s="37">
+      <c r="I7" s="37">
         <v>19300000</v>
       </c>
-      <c r="J2" s="37">
+      <c r="J7" s="37">
         <v>19600000</v>
       </c>
-      <c r="K2" s="37">
+      <c r="K7" s="37">
         <v>19900000</v>
       </c>
-      <c r="L2" s="37">
-        <f>AVERAGE(J2:K2)</f>
-        <v>19750000</v>
-      </c>
-      <c r="M2" s="37">
-        <f t="shared" ref="M2:P2" si="0">AVERAGE(K2:L2)</f>
-        <v>19825000</v>
-      </c>
-      <c r="N2" s="37">
-        <f t="shared" si="0"/>
-        <v>19787500</v>
-      </c>
-      <c r="O2" s="37">
-        <f t="shared" si="0"/>
-        <v>19806250</v>
-      </c>
-      <c r="P2" s="37">
-        <f t="shared" si="0"/>
-        <v>19796875</v>
-      </c>
-      <c r="Q2" s="37">
-        <f t="shared" ref="Q2:Q18" si="1">AVERAGE(O2:P2)</f>
-        <v>19801562.5</v>
-      </c>
-      <c r="R2" s="37">
-        <f t="shared" ref="R2:R18" si="2">AVERAGE(P2:Q2)</f>
-        <v>19799218.75</v>
-      </c>
-      <c r="S2" s="37">
-        <f t="shared" ref="S2:S18" si="3">AVERAGE(Q2:R2)</f>
-        <v>19800390.625</v>
-      </c>
-      <c r="T2" s="37">
-        <f t="shared" ref="T2:T18" si="4">AVERAGE(R2:S2)</f>
-        <v>19799804.6875</v>
-      </c>
-      <c r="U2" s="37">
-        <f t="shared" ref="U2:U18" si="5">AVERAGE(S2:T2)</f>
-        <v>19800097.65625</v>
-      </c>
-      <c r="V2" s="37">
-        <f t="shared" ref="V2:V18" si="6">AVERAGE(T2:U2)</f>
-        <v>19799951.171875</v>
-      </c>
-      <c r="W2" s="37">
-        <f t="shared" ref="W2:W18" si="7">AVERAGE(U2:V2)</f>
-        <v>19800024.4140625</v>
-      </c>
-      <c r="X2" s="37">
-        <f t="shared" ref="X2:X18" si="8">AVERAGE(V2:W2)</f>
-        <v>19799987.79296875</v>
-      </c>
-      <c r="Y2" s="37">
-        <f t="shared" ref="Y2:Y18" si="9">AVERAGE(W2:X2)</f>
-        <v>19800006.103515625</v>
-      </c>
-      <c r="Z2" s="37">
-        <f t="shared" ref="Z2:Z18" si="10">AVERAGE(X2:Y2)</f>
-        <v>19799996.948242188</v>
-      </c>
-      <c r="AA2" s="37">
-        <f t="shared" ref="AA2:AA18" si="11">AVERAGE(Y2:Z2)</f>
-        <v>19800001.525878906</v>
-      </c>
-      <c r="AB2" s="37">
-        <f t="shared" ref="AB2:AB18" si="12">AVERAGE(Z2:AA2)</f>
-        <v>19799999.237060547</v>
-      </c>
-      <c r="AC2" s="37">
-        <f t="shared" ref="AC2:AC18" si="13">AVERAGE(AA2:AB2)</f>
-        <v>19800000.381469727</v>
-      </c>
-      <c r="AD2" s="37">
-        <f t="shared" ref="AD2:AD18" si="14">AVERAGE(AB2:AC2)</f>
-        <v>19799999.809265137</v>
-      </c>
-      <c r="AE2" s="37">
-        <f t="shared" ref="AE2:AE18" si="15">AVERAGE(AC2:AD2)</f>
-        <v>19800000.095367432</v>
-      </c>
-      <c r="AF2" s="37">
-        <f t="shared" ref="AF2:AF18" si="16">AVERAGE(AD2:AE2)</f>
-        <v>19799999.952316284</v>
-      </c>
-      <c r="AG2" s="37">
-        <f t="shared" ref="AG2:AG18" si="17">AVERAGE(AE2:AF2)</f>
-        <v>19800000.023841858</v>
-      </c>
-      <c r="AH2" s="37">
-        <f t="shared" ref="AH2:AH18" si="18">AVERAGE(AF2:AG2)</f>
-        <v>19799999.988079071</v>
-      </c>
-      <c r="AI2" s="37">
-        <f t="shared" ref="AI2:AI18" si="19">AVERAGE(AG2:AH2)</f>
-        <v>19800000.005960464</v>
-      </c>
-      <c r="AJ2" s="37">
-        <f t="shared" ref="AJ2:AJ18" si="20">AVERAGE(AH2:AI2)</f>
-        <v>19799999.997019768</v>
-      </c>
-      <c r="AK2" s="37">
-        <f t="shared" ref="AK2:AK18" si="21">AVERAGE(AI2:AJ2)</f>
-        <v>19800000.001490116</v>
-      </c>
-      <c r="AL2" s="37">
-        <f t="shared" ref="AL2:AL18" si="22">AVERAGE(AJ2:AK2)</f>
-        <v>19799999.999254942</v>
-      </c>
-      <c r="AM2" s="37">
-        <f t="shared" ref="AM2:AM18" si="23">AVERAGE(AK2:AL2)</f>
-        <v>19800000.000372529</v>
-      </c>
-      <c r="AN2" s="37">
-        <f t="shared" ref="AN2:AN18" si="24">AVERAGE(AL2:AM2)</f>
-        <v>19799999.999813735</v>
-      </c>
-      <c r="AO2" s="37">
-        <f t="shared" ref="AO2:AO18" si="25">AVERAGE(AM2:AN2)</f>
-        <v>19800000.000093132</v>
-      </c>
-      <c r="AP2" s="37">
-        <f t="shared" ref="AP2:AP18" si="26">AVERAGE(AN2:AO2)</f>
-        <v>19799999.999953434</v>
-      </c>
-      <c r="AQ2" s="37">
-        <f t="shared" ref="AQ2:AQ18" si="27">AVERAGE(AO2:AP2)</f>
-        <v>19800000.000023283</v>
-      </c>
-      <c r="AR2" s="37">
-        <f t="shared" ref="AR2:AR18" si="28">AVERAGE(AP2:AQ2)</f>
-        <v>19799999.999988358</v>
-      </c>
-      <c r="AS2" s="37">
-        <f t="shared" ref="AS2:AS18" si="29">AVERAGE(AQ2:AR2)</f>
-        <v>19800000.000005819</v>
-      </c>
-      <c r="AT2" s="37">
-        <f t="shared" ref="AT2:AT18" si="30">AVERAGE(AR2:AS2)</f>
-        <v>19799999.999997087</v>
-      </c>
-      <c r="AU2" s="37">
-        <f t="shared" ref="AU2:AU18" si="31">AVERAGE(AS2:AT2)</f>
-        <v>19800000.000001453</v>
-      </c>
-      <c r="AV2" s="37">
-        <f t="shared" ref="AV2:AV18" si="32">AVERAGE(AT2:AU2)</f>
-        <v>19799999.99999927</v>
-      </c>
-      <c r="AW2" s="37">
-        <f t="shared" ref="AW2:AW18" si="33">AVERAGE(AU2:AV2)</f>
-        <v>19800000.000000361</v>
-      </c>
-      <c r="AX2" s="37">
-        <f t="shared" ref="AX2:AX18" si="34">AVERAGE(AV2:AW2)</f>
-        <v>19799999.999999814</v>
-      </c>
-      <c r="AY2" s="37">
-        <f t="shared" ref="AY2:AY18" si="35">AVERAGE(AW2:AX2)</f>
-        <v>19800000.000000089</v>
-      </c>
-    </row>
-    <row r="3" spans="1:51" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>140</v>
       </c>
-      <c r="B3" s="37">
-        <v>24300000</v>
-      </c>
-      <c r="C3" s="37">
-        <v>26300000</v>
-      </c>
-      <c r="D3" s="37">
-        <v>26500000</v>
-      </c>
-      <c r="E3" s="37">
-        <v>25000000</v>
-      </c>
-      <c r="F3" s="37">
-        <v>24900000</v>
-      </c>
-      <c r="G3" s="37">
-        <v>24700000</v>
-      </c>
-      <c r="H3" s="37">
-        <v>25000000</v>
-      </c>
-      <c r="I3" s="37">
-        <v>24800000</v>
-      </c>
-      <c r="J3" s="37">
-        <v>25100000</v>
-      </c>
-      <c r="K3" s="37">
-        <v>25400000</v>
-      </c>
-      <c r="L3" s="37">
-        <f t="shared" ref="L3:L18" si="36">AVERAGE(J3:K3)</f>
-        <v>25250000</v>
-      </c>
-      <c r="M3" s="37">
-        <f t="shared" ref="M3:M18" si="37">AVERAGE(K3:L3)</f>
-        <v>25325000</v>
-      </c>
-      <c r="N3" s="37">
-        <f t="shared" ref="N3:N18" si="38">AVERAGE(L3:M3)</f>
-        <v>25287500</v>
-      </c>
-      <c r="O3" s="37">
-        <f t="shared" ref="O3:O18" si="39">AVERAGE(M3:N3)</f>
-        <v>25306250</v>
-      </c>
-      <c r="P3" s="37">
-        <f t="shared" ref="P3:P18" si="40">AVERAGE(N3:O3)</f>
-        <v>25296875</v>
-      </c>
-      <c r="Q3" s="37">
-        <f t="shared" si="1"/>
-        <v>25301562.5</v>
-      </c>
-      <c r="R3" s="37">
-        <f t="shared" si="2"/>
-        <v>25299218.75</v>
-      </c>
-      <c r="S3" s="37">
-        <f t="shared" si="3"/>
-        <v>25300390.625</v>
-      </c>
-      <c r="T3" s="37">
-        <f t="shared" si="4"/>
-        <v>25299804.6875</v>
-      </c>
-      <c r="U3" s="37">
-        <f t="shared" si="5"/>
-        <v>25300097.65625</v>
-      </c>
-      <c r="V3" s="37">
-        <f t="shared" si="6"/>
-        <v>25299951.171875</v>
-      </c>
-      <c r="W3" s="37">
-        <f t="shared" si="7"/>
-        <v>25300024.4140625</v>
-      </c>
-      <c r="X3" s="37">
-        <f t="shared" si="8"/>
-        <v>25299987.79296875</v>
-      </c>
-      <c r="Y3" s="37">
-        <f t="shared" si="9"/>
-        <v>25300006.103515625</v>
-      </c>
-      <c r="Z3" s="37">
-        <f t="shared" si="10"/>
-        <v>25299996.948242188</v>
-      </c>
-      <c r="AA3" s="37">
-        <f t="shared" si="11"/>
-        <v>25300001.525878906</v>
-      </c>
-      <c r="AB3" s="37">
-        <f t="shared" si="12"/>
-        <v>25299999.237060547</v>
-      </c>
-      <c r="AC3" s="37">
-        <f t="shared" si="13"/>
-        <v>25300000.381469727</v>
-      </c>
-      <c r="AD3" s="37">
-        <f t="shared" si="14"/>
-        <v>25299999.809265137</v>
-      </c>
-      <c r="AE3" s="37">
-        <f t="shared" si="15"/>
-        <v>25300000.095367432</v>
-      </c>
-      <c r="AF3" s="37">
-        <f t="shared" si="16"/>
-        <v>25299999.952316284</v>
-      </c>
-      <c r="AG3" s="37">
-        <f t="shared" si="17"/>
-        <v>25300000.023841858</v>
-      </c>
-      <c r="AH3" s="37">
-        <f t="shared" si="18"/>
-        <v>25299999.988079071</v>
-      </c>
-      <c r="AI3" s="37">
-        <f t="shared" si="19"/>
-        <v>25300000.005960464</v>
-      </c>
-      <c r="AJ3" s="37">
-        <f t="shared" si="20"/>
-        <v>25299999.997019768</v>
-      </c>
-      <c r="AK3" s="37">
-        <f t="shared" si="21"/>
-        <v>25300000.001490116</v>
-      </c>
-      <c r="AL3" s="37">
-        <f t="shared" si="22"/>
-        <v>25299999.999254942</v>
-      </c>
-      <c r="AM3" s="37">
-        <f t="shared" si="23"/>
-        <v>25300000.000372529</v>
-      </c>
-      <c r="AN3" s="37">
-        <f t="shared" si="24"/>
-        <v>25299999.999813735</v>
-      </c>
-      <c r="AO3" s="37">
-        <f t="shared" si="25"/>
-        <v>25300000.000093132</v>
-      </c>
-      <c r="AP3" s="37">
-        <f t="shared" si="26"/>
-        <v>25299999.999953434</v>
-      </c>
-      <c r="AQ3" s="37">
-        <f t="shared" si="27"/>
-        <v>25300000.000023283</v>
-      </c>
-      <c r="AR3" s="37">
-        <f t="shared" si="28"/>
-        <v>25299999.999988358</v>
-      </c>
-      <c r="AS3" s="37">
-        <f t="shared" si="29"/>
-        <v>25300000.000005819</v>
-      </c>
-      <c r="AT3" s="37">
-        <f t="shared" si="30"/>
-        <v>25299999.999997087</v>
-      </c>
-      <c r="AU3" s="37">
-        <f t="shared" si="31"/>
-        <v>25300000.000001453</v>
-      </c>
-      <c r="AV3" s="37">
-        <f t="shared" si="32"/>
-        <v>25299999.99999927</v>
-      </c>
-      <c r="AW3" s="37">
-        <f t="shared" si="33"/>
-        <v>25300000.000000361</v>
-      </c>
-      <c r="AX3" s="37">
-        <f t="shared" si="34"/>
-        <v>25299999.999999814</v>
-      </c>
-      <c r="AY3" s="37">
-        <f t="shared" si="35"/>
-        <v>25300000.000000089</v>
-      </c>
-    </row>
-    <row r="4" spans="1:51" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="B8" s="37">
+        <v>243000000</v>
+      </c>
+      <c r="C8" s="37">
+        <v>263000000</v>
+      </c>
+      <c r="D8" s="37">
+        <v>265000000</v>
+      </c>
+      <c r="E8" s="37">
+        <v>250000000</v>
+      </c>
+      <c r="F8" s="37">
+        <v>249000000</v>
+      </c>
+      <c r="G8" s="37">
+        <v>247000000</v>
+      </c>
+      <c r="H8" s="37">
+        <v>250000000</v>
+      </c>
+      <c r="I8" s="37">
+        <v>248000000</v>
+      </c>
+      <c r="J8" s="37">
+        <v>251000000</v>
+      </c>
+      <c r="K8" s="37">
+        <v>254000000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>141</v>
       </c>
-      <c r="B4" s="37">
+      <c r="B9" s="37">
         <v>8000000</v>
       </c>
-      <c r="C4" s="37">
+      <c r="C9" s="37">
         <v>8600000</v>
       </c>
-      <c r="D4" s="37">
+      <c r="D9" s="37">
         <v>8700000</v>
       </c>
-      <c r="E4" s="37">
+      <c r="E9" s="37">
         <v>8400000</v>
       </c>
-      <c r="F4" s="37">
+      <c r="F9" s="37">
         <v>8400000</v>
       </c>
-      <c r="G4" s="37">
+      <c r="G9" s="37">
         <v>8100000</v>
       </c>
-      <c r="H4" s="38">
+      <c r="H9" s="38">
         <v>8300000</v>
       </c>
-      <c r="I4" s="38">
+      <c r="I9" s="38">
         <v>8200000</v>
       </c>
-      <c r="J4" s="38">
+      <c r="J9" s="38">
         <v>8200000</v>
       </c>
-      <c r="K4" s="38">
+      <c r="K9" s="38">
         <v>8200000</v>
       </c>
-      <c r="L4" s="37">
-        <f t="shared" si="36"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>142</v>
+      </c>
+      <c r="B10" s="37">
+        <v>36000000</v>
+      </c>
+      <c r="C10" s="37">
+        <v>39500000</v>
+      </c>
+      <c r="D10" s="37">
+        <v>40500000</v>
+      </c>
+      <c r="E10" s="37">
+        <v>40200000</v>
+      </c>
+      <c r="F10" s="37">
+        <v>41100000</v>
+      </c>
+      <c r="G10" s="37">
+        <v>40500000</v>
+      </c>
+      <c r="H10" s="38">
+        <v>41300000</v>
+      </c>
+      <c r="I10" s="38">
+        <v>40900000</v>
+      </c>
+      <c r="J10" s="38">
+        <v>41200000</v>
+      </c>
+      <c r="K10" s="38">
+        <v>41300000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>143</v>
+      </c>
+      <c r="B11" s="37">
+        <v>8400000</v>
+      </c>
+      <c r="C11" s="37">
+        <v>11200000</v>
+      </c>
+      <c r="D11" s="37">
+        <v>13100000</v>
+      </c>
+      <c r="E11" s="37">
+        <v>13000000</v>
+      </c>
+      <c r="F11" s="37">
+        <v>13000000</v>
+      </c>
+      <c r="G11" s="37">
+        <v>12800000</v>
+      </c>
+      <c r="H11" s="37">
+        <v>13100000</v>
+      </c>
+      <c r="I11" s="37">
+        <v>12900000</v>
+      </c>
+      <c r="J11" s="37">
+        <v>13100000</v>
+      </c>
+      <c r="K11" s="37">
+        <v>13300000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>145</v>
+      </c>
+      <c r="B12" s="37">
+        <v>30000</v>
+      </c>
+      <c r="C12" s="37">
+        <v>25000</v>
+      </c>
+      <c r="D12" s="37">
+        <v>21000</v>
+      </c>
+      <c r="E12" s="38">
+        <v>0</v>
+      </c>
+      <c r="F12" s="38">
+        <v>0</v>
+      </c>
+      <c r="G12" s="38">
+        <v>0</v>
+      </c>
+      <c r="H12" s="38">
+        <v>0</v>
+      </c>
+      <c r="I12" s="38">
+        <v>0</v>
+      </c>
+      <c r="J12" s="38">
+        <v>0</v>
+      </c>
+      <c r="K12" s="38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>146</v>
+      </c>
+      <c r="B13" s="37">
+        <v>8000000</v>
+      </c>
+      <c r="C13" s="37">
+        <v>8600000</v>
+      </c>
+      <c r="D13" s="37">
+        <v>8700000</v>
+      </c>
+      <c r="E13" s="37">
+        <v>8400000</v>
+      </c>
+      <c r="F13" s="37">
+        <v>8400000</v>
+      </c>
+      <c r="G13" s="37">
+        <v>8100000</v>
+      </c>
+      <c r="H13" s="37">
+        <v>8300000</v>
+      </c>
+      <c r="I13" s="37">
         <v>8200000</v>
       </c>
-      <c r="M4" s="37">
-        <f t="shared" si="37"/>
+      <c r="J13" s="37">
         <v>8200000</v>
       </c>
-      <c r="N4" s="37">
-        <f t="shared" si="38"/>
+      <c r="K13" s="37">
         <v>8200000</v>
       </c>
-      <c r="O4" s="37">
-        <f t="shared" si="39"/>
-        <v>8200000</v>
-      </c>
-      <c r="P4" s="37">
-        <f t="shared" si="40"/>
-        <v>8200000</v>
-      </c>
-      <c r="Q4" s="37">
-        <f t="shared" si="1"/>
-        <v>8200000</v>
-      </c>
-      <c r="R4" s="37">
-        <f t="shared" si="2"/>
-        <v>8200000</v>
-      </c>
-      <c r="S4" s="37">
-        <f t="shared" si="3"/>
-        <v>8200000</v>
-      </c>
-      <c r="T4" s="37">
-        <f t="shared" si="4"/>
-        <v>8200000</v>
-      </c>
-      <c r="U4" s="37">
-        <f t="shared" si="5"/>
-        <v>8200000</v>
-      </c>
-      <c r="V4" s="37">
-        <f t="shared" si="6"/>
-        <v>8200000</v>
-      </c>
-      <c r="W4" s="37">
-        <f t="shared" si="7"/>
-        <v>8200000</v>
-      </c>
-      <c r="X4" s="37">
-        <f t="shared" si="8"/>
-        <v>8200000</v>
-      </c>
-      <c r="Y4" s="37">
-        <f t="shared" si="9"/>
-        <v>8200000</v>
-      </c>
-      <c r="Z4" s="37">
-        <f t="shared" si="10"/>
-        <v>8200000</v>
-      </c>
-      <c r="AA4" s="37">
-        <f t="shared" si="11"/>
-        <v>8200000</v>
-      </c>
-      <c r="AB4" s="37">
-        <f t="shared" si="12"/>
-        <v>8200000</v>
-      </c>
-      <c r="AC4" s="37">
-        <f t="shared" si="13"/>
-        <v>8200000</v>
-      </c>
-      <c r="AD4" s="37">
-        <f t="shared" si="14"/>
-        <v>8200000</v>
-      </c>
-      <c r="AE4" s="37">
-        <f t="shared" si="15"/>
-        <v>8200000</v>
-      </c>
-      <c r="AF4" s="37">
-        <f t="shared" si="16"/>
-        <v>8200000</v>
-      </c>
-      <c r="AG4" s="37">
-        <f t="shared" si="17"/>
-        <v>8200000</v>
-      </c>
-      <c r="AH4" s="37">
-        <f t="shared" si="18"/>
-        <v>8200000</v>
-      </c>
-      <c r="AI4" s="37">
-        <f t="shared" si="19"/>
-        <v>8200000</v>
-      </c>
-      <c r="AJ4" s="37">
-        <f t="shared" si="20"/>
-        <v>8200000</v>
-      </c>
-      <c r="AK4" s="37">
-        <f t="shared" si="21"/>
-        <v>8200000</v>
-      </c>
-      <c r="AL4" s="37">
-        <f t="shared" si="22"/>
-        <v>8200000</v>
-      </c>
-      <c r="AM4" s="37">
-        <f t="shared" si="23"/>
-        <v>8200000</v>
-      </c>
-      <c r="AN4" s="37">
-        <f t="shared" si="24"/>
-        <v>8200000</v>
-      </c>
-      <c r="AO4" s="37">
-        <f t="shared" si="25"/>
-        <v>8200000</v>
-      </c>
-      <c r="AP4" s="37">
-        <f t="shared" si="26"/>
-        <v>8200000</v>
-      </c>
-      <c r="AQ4" s="37">
-        <f t="shared" si="27"/>
-        <v>8200000</v>
-      </c>
-      <c r="AR4" s="37">
-        <f t="shared" si="28"/>
-        <v>8200000</v>
-      </c>
-      <c r="AS4" s="37">
-        <f t="shared" si="29"/>
-        <v>8200000</v>
-      </c>
-      <c r="AT4" s="37">
-        <f t="shared" si="30"/>
-        <v>8200000</v>
-      </c>
-      <c r="AU4" s="37">
-        <f t="shared" si="31"/>
-        <v>8200000</v>
-      </c>
-      <c r="AV4" s="37">
-        <f t="shared" si="32"/>
-        <v>8200000</v>
-      </c>
-      <c r="AW4" s="37">
-        <f t="shared" si="33"/>
-        <v>8200000</v>
-      </c>
-      <c r="AX4" s="37">
-        <f t="shared" si="34"/>
-        <v>8200000</v>
-      </c>
-      <c r="AY4" s="37">
-        <f t="shared" si="35"/>
-        <v>8200000</v>
-      </c>
-    </row>
-    <row r="5" spans="1:51" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>142</v>
-      </c>
-      <c r="B5" s="37">
-        <v>36000000</v>
-      </c>
-      <c r="C5" s="37">
-        <v>39500000</v>
-      </c>
-      <c r="D5" s="37">
-        <v>40500000</v>
-      </c>
-      <c r="E5" s="37">
-        <v>40200000</v>
-      </c>
-      <c r="F5" s="37">
-        <v>41100000</v>
-      </c>
-      <c r="G5" s="37">
-        <v>40500000</v>
-      </c>
-      <c r="H5" s="38">
-        <v>41300000</v>
-      </c>
-      <c r="I5" s="38">
-        <v>40900000</v>
-      </c>
-      <c r="J5" s="38">
-        <v>41200000</v>
-      </c>
-      <c r="K5" s="38">
-        <v>41300000</v>
-      </c>
-      <c r="L5" s="37">
-        <f t="shared" si="36"/>
-        <v>41250000</v>
-      </c>
-      <c r="M5" s="37">
-        <f t="shared" si="37"/>
-        <v>41275000</v>
-      </c>
-      <c r="N5" s="37">
-        <f t="shared" si="38"/>
-        <v>41262500</v>
-      </c>
-      <c r="O5" s="37">
-        <f t="shared" si="39"/>
-        <v>41268750</v>
-      </c>
-      <c r="P5" s="37">
-        <f t="shared" si="40"/>
-        <v>41265625</v>
-      </c>
-      <c r="Q5" s="37">
-        <f t="shared" si="1"/>
-        <v>41267187.5</v>
-      </c>
-      <c r="R5" s="37">
-        <f t="shared" si="2"/>
-        <v>41266406.25</v>
-      </c>
-      <c r="S5" s="37">
-        <f t="shared" si="3"/>
-        <v>41266796.875</v>
-      </c>
-      <c r="T5" s="37">
-        <f t="shared" si="4"/>
-        <v>41266601.5625</v>
-      </c>
-      <c r="U5" s="37">
-        <f t="shared" si="5"/>
-        <v>41266699.21875</v>
-      </c>
-      <c r="V5" s="37">
-        <f t="shared" si="6"/>
-        <v>41266650.390625</v>
-      </c>
-      <c r="W5" s="37">
-        <f t="shared" si="7"/>
-        <v>41266674.8046875</v>
-      </c>
-      <c r="X5" s="37">
-        <f t="shared" si="8"/>
-        <v>41266662.59765625</v>
-      </c>
-      <c r="Y5" s="37">
-        <f t="shared" si="9"/>
-        <v>41266668.701171875</v>
-      </c>
-      <c r="Z5" s="37">
-        <f t="shared" si="10"/>
-        <v>41266665.649414063</v>
-      </c>
-      <c r="AA5" s="37">
-        <f t="shared" si="11"/>
-        <v>41266667.175292969</v>
-      </c>
-      <c r="AB5" s="37">
-        <f t="shared" si="12"/>
-        <v>41266666.412353516</v>
-      </c>
-      <c r="AC5" s="37">
-        <f t="shared" si="13"/>
-        <v>41266666.793823242</v>
-      </c>
-      <c r="AD5" s="37">
-        <f t="shared" si="14"/>
-        <v>41266666.603088379</v>
-      </c>
-      <c r="AE5" s="37">
-        <f t="shared" si="15"/>
-        <v>41266666.698455811</v>
-      </c>
-      <c r="AF5" s="37">
-        <f t="shared" si="16"/>
-        <v>41266666.650772095</v>
-      </c>
-      <c r="AG5" s="37">
-        <f t="shared" si="17"/>
-        <v>41266666.674613953</v>
-      </c>
-      <c r="AH5" s="37">
-        <f t="shared" si="18"/>
-        <v>41266666.662693024</v>
-      </c>
-      <c r="AI5" s="37">
-        <f t="shared" si="19"/>
-        <v>41266666.668653488</v>
-      </c>
-      <c r="AJ5" s="37">
-        <f t="shared" si="20"/>
-        <v>41266666.665673256</v>
-      </c>
-      <c r="AK5" s="37">
-        <f t="shared" si="21"/>
-        <v>41266666.667163372</v>
-      </c>
-      <c r="AL5" s="37">
-        <f t="shared" si="22"/>
-        <v>41266666.666418314</v>
-      </c>
-      <c r="AM5" s="37">
-        <f t="shared" si="23"/>
-        <v>41266666.666790843</v>
-      </c>
-      <c r="AN5" s="37">
-        <f t="shared" si="24"/>
-        <v>41266666.666604578</v>
-      </c>
-      <c r="AO5" s="37">
-        <f t="shared" si="25"/>
-        <v>41266666.666697711</v>
-      </c>
-      <c r="AP5" s="37">
-        <f t="shared" si="26"/>
-        <v>41266666.666651145</v>
-      </c>
-      <c r="AQ5" s="37">
-        <f t="shared" si="27"/>
-        <v>41266666.666674428</v>
-      </c>
-      <c r="AR5" s="37">
-        <f t="shared" si="28"/>
-        <v>41266666.666662782</v>
-      </c>
-      <c r="AS5" s="37">
-        <f t="shared" si="29"/>
-        <v>41266666.666668609</v>
-      </c>
-      <c r="AT5" s="37">
-        <f t="shared" si="30"/>
-        <v>41266666.666665696</v>
-      </c>
-      <c r="AU5" s="37">
-        <f t="shared" si="31"/>
-        <v>41266666.666667148</v>
-      </c>
-      <c r="AV5" s="37">
-        <f t="shared" si="32"/>
-        <v>41266666.666666418</v>
-      </c>
-      <c r="AW5" s="37">
-        <f t="shared" si="33"/>
-        <v>41266666.666666783</v>
-      </c>
-      <c r="AX5" s="37">
-        <f t="shared" si="34"/>
-        <v>41266666.666666597</v>
-      </c>
-      <c r="AY5" s="37">
-        <f t="shared" si="35"/>
-        <v>41266666.666666687</v>
-      </c>
-    </row>
-    <row r="6" spans="1:51" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>143</v>
-      </c>
-      <c r="B6" s="37">
-        <v>8400000</v>
-      </c>
-      <c r="C6" s="37">
-        <v>11200000</v>
-      </c>
-      <c r="D6" s="37">
-        <v>13100000</v>
-      </c>
-      <c r="E6" s="37">
-        <v>13000000</v>
-      </c>
-      <c r="F6" s="37">
-        <v>13000000</v>
-      </c>
-      <c r="G6" s="37">
-        <v>12800000</v>
-      </c>
-      <c r="H6" s="37">
-        <v>13100000</v>
-      </c>
-      <c r="I6" s="37">
-        <v>12900000</v>
-      </c>
-      <c r="J6" s="37">
-        <v>13100000</v>
-      </c>
-      <c r="K6" s="37">
-        <v>13300000</v>
-      </c>
-      <c r="L6" s="37">
-        <f t="shared" si="36"/>
-        <v>13200000</v>
-      </c>
-      <c r="M6" s="37">
-        <f t="shared" si="37"/>
-        <v>13250000</v>
-      </c>
-      <c r="N6" s="37">
-        <f t="shared" si="38"/>
-        <v>13225000</v>
-      </c>
-      <c r="O6" s="37">
-        <f t="shared" si="39"/>
-        <v>13237500</v>
-      </c>
-      <c r="P6" s="37">
-        <f t="shared" si="40"/>
-        <v>13231250</v>
-      </c>
-      <c r="Q6" s="37">
-        <f t="shared" si="1"/>
-        <v>13234375</v>
-      </c>
-      <c r="R6" s="37">
-        <f t="shared" si="2"/>
-        <v>13232812.5</v>
-      </c>
-      <c r="S6" s="37">
-        <f t="shared" si="3"/>
-        <v>13233593.75</v>
-      </c>
-      <c r="T6" s="37">
-        <f t="shared" si="4"/>
-        <v>13233203.125</v>
-      </c>
-      <c r="U6" s="37">
-        <f t="shared" si="5"/>
-        <v>13233398.4375</v>
-      </c>
-      <c r="V6" s="37">
-        <f t="shared" si="6"/>
-        <v>13233300.78125</v>
-      </c>
-      <c r="W6" s="37">
-        <f t="shared" si="7"/>
-        <v>13233349.609375</v>
-      </c>
-      <c r="X6" s="37">
-        <f t="shared" si="8"/>
-        <v>13233325.1953125</v>
-      </c>
-      <c r="Y6" s="37">
-        <f t="shared" si="9"/>
-        <v>13233337.40234375</v>
-      </c>
-      <c r="Z6" s="37">
-        <f t="shared" si="10"/>
-        <v>13233331.298828125</v>
-      </c>
-      <c r="AA6" s="37">
-        <f t="shared" si="11"/>
-        <v>13233334.350585938</v>
-      </c>
-      <c r="AB6" s="37">
-        <f t="shared" si="12"/>
-        <v>13233332.824707031</v>
-      </c>
-      <c r="AC6" s="37">
-        <f t="shared" si="13"/>
-        <v>13233333.587646484</v>
-      </c>
-      <c r="AD6" s="37">
-        <f t="shared" si="14"/>
-        <v>13233333.206176758</v>
-      </c>
-      <c r="AE6" s="37">
-        <f t="shared" si="15"/>
-        <v>13233333.396911621</v>
-      </c>
-      <c r="AF6" s="37">
-        <f t="shared" si="16"/>
-        <v>13233333.301544189</v>
-      </c>
-      <c r="AG6" s="37">
-        <f t="shared" si="17"/>
-        <v>13233333.349227905</v>
-      </c>
-      <c r="AH6" s="37">
-        <f t="shared" si="18"/>
-        <v>13233333.325386047</v>
-      </c>
-      <c r="AI6" s="37">
-        <f t="shared" si="19"/>
-        <v>13233333.337306976</v>
-      </c>
-      <c r="AJ6" s="37">
-        <f t="shared" si="20"/>
-        <v>13233333.331346512</v>
-      </c>
-      <c r="AK6" s="37">
-        <f t="shared" si="21"/>
-        <v>13233333.334326744</v>
-      </c>
-      <c r="AL6" s="37">
-        <f t="shared" si="22"/>
-        <v>13233333.332836628</v>
-      </c>
-      <c r="AM6" s="37">
-        <f t="shared" si="23"/>
-        <v>13233333.333581686</v>
-      </c>
-      <c r="AN6" s="37">
-        <f t="shared" si="24"/>
-        <v>13233333.333209157</v>
-      </c>
-      <c r="AO6" s="37">
-        <f t="shared" si="25"/>
-        <v>13233333.333395422</v>
-      </c>
-      <c r="AP6" s="37">
-        <f t="shared" si="26"/>
-        <v>13233333.333302289</v>
-      </c>
-      <c r="AQ6" s="37">
-        <f t="shared" si="27"/>
-        <v>13233333.333348855</v>
-      </c>
-      <c r="AR6" s="37">
-        <f t="shared" si="28"/>
-        <v>13233333.333325572</v>
-      </c>
-      <c r="AS6" s="37">
-        <f t="shared" si="29"/>
-        <v>13233333.333337214</v>
-      </c>
-      <c r="AT6" s="37">
-        <f t="shared" si="30"/>
-        <v>13233333.333331393</v>
-      </c>
-      <c r="AU6" s="37">
-        <f t="shared" si="31"/>
-        <v>13233333.333334304</v>
-      </c>
-      <c r="AV6" s="37">
-        <f t="shared" si="32"/>
-        <v>13233333.333332848</v>
-      </c>
-      <c r="AW6" s="37">
-        <f t="shared" si="33"/>
-        <v>13233333.333333576</v>
-      </c>
-      <c r="AX6" s="37">
-        <f t="shared" si="34"/>
-        <v>13233333.333333213</v>
-      </c>
-      <c r="AY6" s="37">
-        <f t="shared" si="35"/>
-        <v>13233333.333333395</v>
-      </c>
-    </row>
-    <row r="7" spans="1:51" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>144</v>
-      </c>
-      <c r="B7" s="37">
-        <v>160100000</v>
-      </c>
-      <c r="C7" s="37">
-        <v>140800000</v>
-      </c>
-      <c r="D7" s="37">
-        <v>154800000</v>
-      </c>
-      <c r="E7" s="37">
-        <v>143800000</v>
-      </c>
-      <c r="F7" s="37">
-        <v>147500000</v>
-      </c>
-      <c r="G7" s="37">
-        <v>171200000</v>
-      </c>
-      <c r="H7" s="37">
-        <v>139700000</v>
-      </c>
-      <c r="I7" s="37">
-        <v>172900000</v>
-      </c>
-      <c r="J7" s="37">
-        <v>149300000</v>
-      </c>
-      <c r="K7" s="37">
-        <v>158400000</v>
-      </c>
-      <c r="L7" s="37">
-        <f t="shared" si="36"/>
-        <v>153850000</v>
-      </c>
-      <c r="M7" s="37">
-        <f t="shared" si="37"/>
-        <v>156125000</v>
-      </c>
-      <c r="N7" s="37">
-        <f t="shared" si="38"/>
-        <v>154987500</v>
-      </c>
-      <c r="O7" s="37">
-        <f t="shared" si="39"/>
-        <v>155556250</v>
-      </c>
-      <c r="P7" s="37">
-        <f t="shared" si="40"/>
-        <v>155271875</v>
-      </c>
-      <c r="Q7" s="37">
-        <f t="shared" si="1"/>
-        <v>155414062.5</v>
-      </c>
-      <c r="R7" s="37">
-        <f t="shared" si="2"/>
-        <v>155342968.75</v>
-      </c>
-      <c r="S7" s="37">
-        <f t="shared" si="3"/>
-        <v>155378515.625</v>
-      </c>
-      <c r="T7" s="37">
-        <f t="shared" si="4"/>
-        <v>155360742.1875</v>
-      </c>
-      <c r="U7" s="37">
-        <f t="shared" si="5"/>
-        <v>155369628.90625</v>
-      </c>
-      <c r="V7" s="37">
-        <f t="shared" si="6"/>
-        <v>155365185.546875</v>
-      </c>
-      <c r="W7" s="37">
-        <f t="shared" si="7"/>
-        <v>155367407.2265625</v>
-      </c>
-      <c r="X7" s="37">
-        <f t="shared" si="8"/>
-        <v>155366296.38671875</v>
-      </c>
-      <c r="Y7" s="37">
-        <f t="shared" si="9"/>
-        <v>155366851.80664063</v>
-      </c>
-      <c r="Z7" s="37">
-        <f t="shared" si="10"/>
-        <v>155366574.09667969</v>
-      </c>
-      <c r="AA7" s="37">
-        <f t="shared" si="11"/>
-        <v>155366712.95166016</v>
-      </c>
-      <c r="AB7" s="37">
-        <f t="shared" si="12"/>
-        <v>155366643.52416992</v>
-      </c>
-      <c r="AC7" s="37">
-        <f t="shared" si="13"/>
-        <v>155366678.23791504</v>
-      </c>
-      <c r="AD7" s="37">
-        <f t="shared" si="14"/>
-        <v>155366660.88104248</v>
-      </c>
-      <c r="AE7" s="37">
-        <f t="shared" si="15"/>
-        <v>155366669.55947876</v>
-      </c>
-      <c r="AF7" s="37">
-        <f t="shared" si="16"/>
-        <v>155366665.22026062</v>
-      </c>
-      <c r="AG7" s="37">
-        <f t="shared" si="17"/>
-        <v>155366667.38986969</v>
-      </c>
-      <c r="AH7" s="37">
-        <f t="shared" si="18"/>
-        <v>155366666.30506516</v>
-      </c>
-      <c r="AI7" s="37">
-        <f t="shared" si="19"/>
-        <v>155366666.84746742</v>
-      </c>
-      <c r="AJ7" s="37">
-        <f t="shared" si="20"/>
-        <v>155366666.57626629</v>
-      </c>
-      <c r="AK7" s="37">
-        <f t="shared" si="21"/>
-        <v>155366666.71186686</v>
-      </c>
-      <c r="AL7" s="37">
-        <f t="shared" si="22"/>
-        <v>155366666.64406657</v>
-      </c>
-      <c r="AM7" s="37">
-        <f t="shared" si="23"/>
-        <v>155366666.67796671</v>
-      </c>
-      <c r="AN7" s="37">
-        <f t="shared" si="24"/>
-        <v>155366666.66101664</v>
-      </c>
-      <c r="AO7" s="37">
-        <f t="shared" si="25"/>
-        <v>155366666.66949168</v>
-      </c>
-      <c r="AP7" s="37">
-        <f t="shared" si="26"/>
-        <v>155366666.66525418</v>
-      </c>
-      <c r="AQ7" s="37">
-        <f t="shared" si="27"/>
-        <v>155366666.66737294</v>
-      </c>
-      <c r="AR7" s="37">
-        <f t="shared" si="28"/>
-        <v>155366666.66631356</v>
-      </c>
-      <c r="AS7" s="37">
-        <f t="shared" si="29"/>
-        <v>155366666.66684324</v>
-      </c>
-      <c r="AT7" s="37">
-        <f t="shared" si="30"/>
-        <v>155366666.66657841</v>
-      </c>
-      <c r="AU7" s="37">
-        <f t="shared" si="31"/>
-        <v>155366666.66671082</v>
-      </c>
-      <c r="AV7" s="37">
-        <f t="shared" si="32"/>
-        <v>155366666.66664463</v>
-      </c>
-      <c r="AW7" s="37">
-        <f t="shared" si="33"/>
-        <v>155366666.66667771</v>
-      </c>
-      <c r="AX7" s="37">
-        <f t="shared" si="34"/>
-        <v>155366666.66666117</v>
-      </c>
-      <c r="AY7" s="37">
-        <f t="shared" si="35"/>
-        <v>155366666.66666943</v>
-      </c>
-    </row>
-    <row r="8" spans="1:51" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>145</v>
-      </c>
-      <c r="B8" s="37">
-        <v>30000</v>
-      </c>
-      <c r="C8" s="37">
-        <v>25000</v>
-      </c>
-      <c r="D8" s="37">
-        <v>25000</v>
-      </c>
-      <c r="E8" s="38">
-        <v>0</v>
-      </c>
-      <c r="F8" s="38">
-        <v>0</v>
-      </c>
-      <c r="G8" s="38">
-        <v>0</v>
-      </c>
-      <c r="H8" s="38">
-        <v>0</v>
-      </c>
-      <c r="I8" s="38">
-        <v>0</v>
-      </c>
-      <c r="J8" s="38">
-        <v>0</v>
-      </c>
-      <c r="K8" s="38">
-        <v>0</v>
-      </c>
-      <c r="L8" s="37">
-        <f t="shared" si="36"/>
-        <v>0</v>
-      </c>
-      <c r="M8" s="37">
-        <f t="shared" si="37"/>
-        <v>0</v>
-      </c>
-      <c r="N8" s="37">
-        <f t="shared" si="38"/>
-        <v>0</v>
-      </c>
-      <c r="O8" s="37">
-        <f t="shared" si="39"/>
-        <v>0</v>
-      </c>
-      <c r="P8" s="37">
-        <f t="shared" si="40"/>
-        <v>0</v>
-      </c>
-      <c r="Q8" s="37">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="R8" s="37">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="S8" s="37">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="T8" s="37">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="U8" s="37">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="V8" s="37">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="W8" s="37">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="X8" s="37">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="Y8" s="37">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="Z8" s="37">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="AA8" s="37">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="AB8" s="37">
-        <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="AC8" s="37">
-        <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-      <c r="AD8" s="37">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="AE8" s="37">
-        <f t="shared" si="15"/>
-        <v>0</v>
-      </c>
-      <c r="AF8" s="37">
-        <f t="shared" si="16"/>
-        <v>0</v>
-      </c>
-      <c r="AG8" s="37">
-        <f t="shared" si="17"/>
-        <v>0</v>
-      </c>
-      <c r="AH8" s="37">
-        <f t="shared" si="18"/>
-        <v>0</v>
-      </c>
-      <c r="AI8" s="37">
-        <f t="shared" si="19"/>
-        <v>0</v>
-      </c>
-      <c r="AJ8" s="37">
-        <f t="shared" si="20"/>
-        <v>0</v>
-      </c>
-      <c r="AK8" s="37">
-        <f t="shared" si="21"/>
-        <v>0</v>
-      </c>
-      <c r="AL8" s="37">
-        <f t="shared" si="22"/>
-        <v>0</v>
-      </c>
-      <c r="AM8" s="37">
-        <f t="shared" si="23"/>
-        <v>0</v>
-      </c>
-      <c r="AN8" s="37">
-        <f t="shared" si="24"/>
-        <v>0</v>
-      </c>
-      <c r="AO8" s="37">
-        <f t="shared" si="25"/>
-        <v>0</v>
-      </c>
-      <c r="AP8" s="37">
-        <f t="shared" si="26"/>
-        <v>0</v>
-      </c>
-      <c r="AQ8" s="37">
-        <f t="shared" si="27"/>
-        <v>0</v>
-      </c>
-      <c r="AR8" s="37">
-        <f t="shared" si="28"/>
-        <v>0</v>
-      </c>
-      <c r="AS8" s="37">
-        <f t="shared" si="29"/>
-        <v>0</v>
-      </c>
-      <c r="AT8" s="37">
-        <f t="shared" si="30"/>
-        <v>0</v>
-      </c>
-      <c r="AU8" s="37">
-        <f t="shared" si="31"/>
-        <v>0</v>
-      </c>
-      <c r="AV8" s="37">
-        <f t="shared" si="32"/>
-        <v>0</v>
-      </c>
-      <c r="AW8" s="37">
-        <f t="shared" si="33"/>
-        <v>0</v>
-      </c>
-      <c r="AX8" s="37">
-        <f t="shared" si="34"/>
-        <v>0</v>
-      </c>
-      <c r="AY8" s="37">
-        <f t="shared" si="35"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:51" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>116</v>
-      </c>
-      <c r="B9" s="37">
-        <v>1646350000</v>
-      </c>
-      <c r="C9" s="37">
-        <v>1824950000</v>
-      </c>
-      <c r="D9" s="37">
-        <v>1975050000</v>
-      </c>
-      <c r="E9" s="37">
-        <v>2271450000</v>
-      </c>
-      <c r="F9" s="37">
-        <v>2472850000</v>
-      </c>
-      <c r="G9" s="37">
-        <v>2252450000</v>
-      </c>
-      <c r="H9" s="37">
-        <v>2138450000</v>
-      </c>
-      <c r="I9" s="37">
-        <v>2088100000</v>
-      </c>
-      <c r="J9" s="37">
-        <v>2047250000</v>
-      </c>
-      <c r="K9" s="37">
-        <v>2069100000</v>
-      </c>
-      <c r="L9" s="37">
-        <f t="shared" si="36"/>
-        <v>2058175000</v>
-      </c>
-      <c r="M9" s="37">
-        <f t="shared" si="37"/>
-        <v>2063637500</v>
-      </c>
-      <c r="N9" s="37">
-        <f t="shared" si="38"/>
-        <v>2060906250</v>
-      </c>
-      <c r="O9" s="37">
-        <f t="shared" si="39"/>
-        <v>2062271875</v>
-      </c>
-      <c r="P9" s="37">
-        <f t="shared" si="40"/>
-        <v>2061589062.5</v>
-      </c>
-      <c r="Q9" s="37">
-        <f t="shared" si="1"/>
-        <v>2061930468.75</v>
-      </c>
-      <c r="R9" s="37">
-        <f t="shared" si="2"/>
-        <v>2061759765.625</v>
-      </c>
-      <c r="S9" s="37">
-        <f t="shared" si="3"/>
-        <v>2061845117.1875</v>
-      </c>
-      <c r="T9" s="37">
-        <f t="shared" si="4"/>
-        <v>2061802441.40625</v>
-      </c>
-      <c r="U9" s="37">
-        <f t="shared" si="5"/>
-        <v>2061823779.296875</v>
-      </c>
-      <c r="V9" s="37">
-        <f t="shared" si="6"/>
-        <v>2061813110.3515625</v>
-      </c>
-      <c r="W9" s="37">
-        <f t="shared" si="7"/>
-        <v>2061818444.8242188</v>
-      </c>
-      <c r="X9" s="37">
-        <f t="shared" si="8"/>
-        <v>2061815777.5878906</v>
-      </c>
-      <c r="Y9" s="37">
-        <f t="shared" si="9"/>
-        <v>2061817111.2060547</v>
-      </c>
-      <c r="Z9" s="37">
-        <f t="shared" si="10"/>
-        <v>2061816444.3969727</v>
-      </c>
-      <c r="AA9" s="37">
-        <f t="shared" si="11"/>
-        <v>2061816777.8015137</v>
-      </c>
-      <c r="AB9" s="37">
-        <f t="shared" si="12"/>
-        <v>2061816611.0992432</v>
-      </c>
-      <c r="AC9" s="37">
-        <f t="shared" si="13"/>
-        <v>2061816694.4503784</v>
-      </c>
-      <c r="AD9" s="37">
-        <f t="shared" si="14"/>
-        <v>2061816652.7748108</v>
-      </c>
-      <c r="AE9" s="37">
-        <f t="shared" si="15"/>
-        <v>2061816673.6125946</v>
-      </c>
-      <c r="AF9" s="37">
-        <f t="shared" si="16"/>
-        <v>2061816663.1937027</v>
-      </c>
-      <c r="AG9" s="37">
-        <f t="shared" si="17"/>
-        <v>2061816668.4031487</v>
-      </c>
-      <c r="AH9" s="37">
-        <f t="shared" si="18"/>
-        <v>2061816665.7984257</v>
-      </c>
-      <c r="AI9" s="37">
-        <f t="shared" si="19"/>
-        <v>2061816667.1007872</v>
-      </c>
-      <c r="AJ9" s="37">
-        <f t="shared" si="20"/>
-        <v>2061816666.4496064</v>
-      </c>
-      <c r="AK9" s="37">
-        <f t="shared" si="21"/>
-        <v>2061816666.7751968</v>
-      </c>
-      <c r="AL9" s="37">
-        <f t="shared" si="22"/>
-        <v>2061816666.6124015</v>
-      </c>
-      <c r="AM9" s="37">
-        <f t="shared" si="23"/>
-        <v>2061816666.693799</v>
-      </c>
-      <c r="AN9" s="37">
-        <f t="shared" si="24"/>
-        <v>2061816666.6531003</v>
-      </c>
-      <c r="AO9" s="37">
-        <f t="shared" si="25"/>
-        <v>2061816666.6734495</v>
-      </c>
-      <c r="AP9" s="37">
-        <f t="shared" si="26"/>
-        <v>2061816666.6632748</v>
-      </c>
-      <c r="AQ9" s="37">
-        <f t="shared" si="27"/>
-        <v>2061816666.6683621</v>
-      </c>
-      <c r="AR9" s="37">
-        <f t="shared" si="28"/>
-        <v>2061816666.6658185</v>
-      </c>
-      <c r="AS9" s="37">
-        <f t="shared" si="29"/>
-        <v>2061816666.6670904</v>
-      </c>
-      <c r="AT9" s="37">
-        <f t="shared" si="30"/>
-        <v>2061816666.6664543</v>
-      </c>
-      <c r="AU9" s="37">
-        <f t="shared" si="31"/>
-        <v>2061816666.6667724</v>
-      </c>
-      <c r="AV9" s="37">
-        <f t="shared" si="32"/>
-        <v>2061816666.6666133</v>
-      </c>
-      <c r="AW9" s="37">
-        <f t="shared" si="33"/>
-        <v>2061816666.6666927</v>
-      </c>
-      <c r="AX9" s="37">
-        <f t="shared" si="34"/>
-        <v>2061816666.6666532</v>
-      </c>
-      <c r="AY9" s="37">
-        <f t="shared" si="35"/>
-        <v>2061816666.6666729</v>
-      </c>
-    </row>
-    <row r="10" spans="1:51" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>146</v>
-      </c>
-      <c r="B10" s="37">
-        <v>8000000</v>
-      </c>
-      <c r="C10" s="37">
-        <v>8600000</v>
-      </c>
-      <c r="D10" s="37">
-        <v>8700000</v>
-      </c>
-      <c r="E10" s="37">
-        <v>8400000</v>
-      </c>
-      <c r="F10" s="37">
-        <v>8400000</v>
-      </c>
-      <c r="G10" s="37">
-        <v>8100000</v>
-      </c>
-      <c r="H10" s="37">
-        <v>8300000</v>
-      </c>
-      <c r="I10" s="37">
-        <v>8200000</v>
-      </c>
-      <c r="J10" s="37">
-        <v>8200000</v>
-      </c>
-      <c r="K10" s="37">
-        <v>8200000</v>
-      </c>
-      <c r="L10" s="37">
-        <f t="shared" si="36"/>
-        <v>8200000</v>
-      </c>
-      <c r="M10" s="37">
-        <f t="shared" si="37"/>
-        <v>8200000</v>
-      </c>
-      <c r="N10" s="37">
-        <f t="shared" si="38"/>
-        <v>8200000</v>
-      </c>
-      <c r="O10" s="37">
-        <f t="shared" si="39"/>
-        <v>8200000</v>
-      </c>
-      <c r="P10" s="37">
-        <f t="shared" si="40"/>
-        <v>8200000</v>
-      </c>
-      <c r="Q10" s="37">
-        <f t="shared" si="1"/>
-        <v>8200000</v>
-      </c>
-      <c r="R10" s="37">
-        <f t="shared" si="2"/>
-        <v>8200000</v>
-      </c>
-      <c r="S10" s="37">
-        <f t="shared" si="3"/>
-        <v>8200000</v>
-      </c>
-      <c r="T10" s="37">
-        <f t="shared" si="4"/>
-        <v>8200000</v>
-      </c>
-      <c r="U10" s="37">
-        <f t="shared" si="5"/>
-        <v>8200000</v>
-      </c>
-      <c r="V10" s="37">
-        <f t="shared" si="6"/>
-        <v>8200000</v>
-      </c>
-      <c r="W10" s="37">
-        <f t="shared" si="7"/>
-        <v>8200000</v>
-      </c>
-      <c r="X10" s="37">
-        <f t="shared" si="8"/>
-        <v>8200000</v>
-      </c>
-      <c r="Y10" s="37">
-        <f t="shared" si="9"/>
-        <v>8200000</v>
-      </c>
-      <c r="Z10" s="37">
-        <f t="shared" si="10"/>
-        <v>8200000</v>
-      </c>
-      <c r="AA10" s="37">
-        <f t="shared" si="11"/>
-        <v>8200000</v>
-      </c>
-      <c r="AB10" s="37">
-        <f t="shared" si="12"/>
-        <v>8200000</v>
-      </c>
-      <c r="AC10" s="37">
-        <f t="shared" si="13"/>
-        <v>8200000</v>
-      </c>
-      <c r="AD10" s="37">
-        <f t="shared" si="14"/>
-        <v>8200000</v>
-      </c>
-      <c r="AE10" s="37">
-        <f t="shared" si="15"/>
-        <v>8200000</v>
-      </c>
-      <c r="AF10" s="37">
-        <f t="shared" si="16"/>
-        <v>8200000</v>
-      </c>
-      <c r="AG10" s="37">
-        <f t="shared" si="17"/>
-        <v>8200000</v>
-      </c>
-      <c r="AH10" s="37">
-        <f t="shared" si="18"/>
-        <v>8200000</v>
-      </c>
-      <c r="AI10" s="37">
-        <f t="shared" si="19"/>
-        <v>8200000</v>
-      </c>
-      <c r="AJ10" s="37">
-        <f t="shared" si="20"/>
-        <v>8200000</v>
-      </c>
-      <c r="AK10" s="37">
-        <f t="shared" si="21"/>
-        <v>8200000</v>
-      </c>
-      <c r="AL10" s="37">
-        <f t="shared" si="22"/>
-        <v>8200000</v>
-      </c>
-      <c r="AM10" s="37">
-        <f t="shared" si="23"/>
-        <v>8200000</v>
-      </c>
-      <c r="AN10" s="37">
-        <f t="shared" si="24"/>
-        <v>8200000</v>
-      </c>
-      <c r="AO10" s="37">
-        <f t="shared" si="25"/>
-        <v>8200000</v>
-      </c>
-      <c r="AP10" s="37">
-        <f t="shared" si="26"/>
-        <v>8200000</v>
-      </c>
-      <c r="AQ10" s="37">
-        <f t="shared" si="27"/>
-        <v>8200000</v>
-      </c>
-      <c r="AR10" s="37">
-        <f t="shared" si="28"/>
-        <v>8200000</v>
-      </c>
-      <c r="AS10" s="37">
-        <f t="shared" si="29"/>
-        <v>8200000</v>
-      </c>
-      <c r="AT10" s="37">
-        <f t="shared" si="30"/>
-        <v>8200000</v>
-      </c>
-      <c r="AU10" s="37">
-        <f t="shared" si="31"/>
-        <v>8200000</v>
-      </c>
-      <c r="AV10" s="37">
-        <f t="shared" si="32"/>
-        <v>8200000</v>
-      </c>
-      <c r="AW10" s="37">
-        <f t="shared" si="33"/>
-        <v>8200000</v>
-      </c>
-      <c r="AX10" s="37">
-        <f t="shared" si="34"/>
-        <v>8200000</v>
-      </c>
-      <c r="AY10" s="37">
-        <f t="shared" si="35"/>
-        <v>8200000</v>
-      </c>
-    </row>
-    <row r="11" spans="1:51" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>147</v>
       </c>
-      <c r="B11" s="37">
-        <v>60600000</v>
-      </c>
-      <c r="C11" s="37">
-        <v>74600000</v>
-      </c>
-      <c r="D11" s="37">
-        <v>83000000</v>
-      </c>
-      <c r="E11" s="37">
-        <v>81300000</v>
-      </c>
-      <c r="F11" s="37">
-        <v>81100000</v>
-      </c>
-      <c r="G11" s="37">
-        <v>79800000</v>
-      </c>
-      <c r="H11" s="37">
-        <v>81100000</v>
-      </c>
-      <c r="I11" s="37">
-        <v>79900000</v>
-      </c>
-      <c r="J11" s="37">
-        <v>81200000</v>
-      </c>
-      <c r="K11" s="37">
-        <v>82300000</v>
-      </c>
-      <c r="L11" s="37">
-        <f t="shared" si="36"/>
-        <v>81750000</v>
-      </c>
-      <c r="M11" s="37">
-        <f t="shared" si="37"/>
-        <v>82025000</v>
-      </c>
-      <c r="N11" s="37">
-        <f t="shared" si="38"/>
-        <v>81887500</v>
-      </c>
-      <c r="O11" s="37">
-        <f t="shared" si="39"/>
-        <v>81956250</v>
-      </c>
-      <c r="P11" s="37">
-        <f t="shared" si="40"/>
-        <v>81921875</v>
-      </c>
-      <c r="Q11" s="37">
-        <f t="shared" si="1"/>
-        <v>81939062.5</v>
-      </c>
-      <c r="R11" s="37">
-        <f t="shared" si="2"/>
-        <v>81930468.75</v>
-      </c>
-      <c r="S11" s="37">
-        <f t="shared" si="3"/>
-        <v>81934765.625</v>
-      </c>
-      <c r="T11" s="37">
-        <f t="shared" si="4"/>
-        <v>81932617.1875</v>
-      </c>
-      <c r="U11" s="37">
-        <f t="shared" si="5"/>
-        <v>81933691.40625</v>
-      </c>
-      <c r="V11" s="37">
-        <f t="shared" si="6"/>
-        <v>81933154.296875</v>
-      </c>
-      <c r="W11" s="37">
-        <f t="shared" si="7"/>
-        <v>81933422.8515625</v>
-      </c>
-      <c r="X11" s="37">
-        <f t="shared" si="8"/>
-        <v>81933288.57421875</v>
-      </c>
-      <c r="Y11" s="37">
-        <f t="shared" si="9"/>
-        <v>81933355.712890625</v>
-      </c>
-      <c r="Z11" s="37">
-        <f t="shared" si="10"/>
-        <v>81933322.143554688</v>
-      </c>
-      <c r="AA11" s="37">
-        <f t="shared" si="11"/>
-        <v>81933338.928222656</v>
-      </c>
-      <c r="AB11" s="37">
-        <f t="shared" si="12"/>
-        <v>81933330.535888672</v>
-      </c>
-      <c r="AC11" s="37">
-        <f t="shared" si="13"/>
-        <v>81933334.732055664</v>
-      </c>
-      <c r="AD11" s="37">
-        <f t="shared" si="14"/>
-        <v>81933332.633972168</v>
-      </c>
-      <c r="AE11" s="37">
-        <f t="shared" si="15"/>
-        <v>81933333.683013916</v>
-      </c>
-      <c r="AF11" s="37">
-        <f t="shared" si="16"/>
-        <v>81933333.158493042</v>
-      </c>
-      <c r="AG11" s="37">
-        <f t="shared" si="17"/>
-        <v>81933333.420753479</v>
-      </c>
-      <c r="AH11" s="37">
-        <f t="shared" si="18"/>
-        <v>81933333.28962326</v>
-      </c>
-      <c r="AI11" s="37">
-        <f t="shared" si="19"/>
-        <v>81933333.35518837</v>
-      </c>
-      <c r="AJ11" s="37">
-        <f t="shared" si="20"/>
-        <v>81933333.322405815</v>
-      </c>
-      <c r="AK11" s="37">
-        <f t="shared" si="21"/>
-        <v>81933333.338797092</v>
-      </c>
-      <c r="AL11" s="37">
-        <f t="shared" si="22"/>
-        <v>81933333.330601454</v>
-      </c>
-      <c r="AM11" s="37">
-        <f t="shared" si="23"/>
-        <v>81933333.334699273</v>
-      </c>
-      <c r="AN11" s="37">
-        <f t="shared" si="24"/>
-        <v>81933333.332650363</v>
-      </c>
-      <c r="AO11" s="37">
-        <f t="shared" si="25"/>
-        <v>81933333.333674818</v>
-      </c>
-      <c r="AP11" s="37">
-        <f t="shared" si="26"/>
-        <v>81933333.333162591</v>
-      </c>
-      <c r="AQ11" s="37">
-        <f t="shared" si="27"/>
-        <v>81933333.333418697</v>
-      </c>
-      <c r="AR11" s="37">
-        <f t="shared" si="28"/>
-        <v>81933333.333290637</v>
-      </c>
-      <c r="AS11" s="37">
-        <f t="shared" si="29"/>
-        <v>81933333.333354667</v>
-      </c>
-      <c r="AT11" s="37">
-        <f t="shared" si="30"/>
-        <v>81933333.333322644</v>
-      </c>
-      <c r="AU11" s="37">
-        <f t="shared" si="31"/>
-        <v>81933333.333338648</v>
-      </c>
-      <c r="AV11" s="37">
-        <f t="shared" si="32"/>
-        <v>81933333.333330646</v>
-      </c>
-      <c r="AW11" s="37">
-        <f t="shared" si="33"/>
-        <v>81933333.333334655</v>
-      </c>
-      <c r="AX11" s="37">
-        <f t="shared" si="34"/>
-        <v>81933333.333332658</v>
-      </c>
-      <c r="AY11" s="37">
-        <f t="shared" si="35"/>
-        <v>81933333.333333656</v>
-      </c>
-    </row>
-    <row r="12" spans="1:51" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>148</v>
-      </c>
-      <c r="B12" s="37">
-        <v>3100000</v>
-      </c>
-      <c r="C12" s="37">
-        <v>3100000</v>
-      </c>
-      <c r="D12" s="37">
-        <v>4500000</v>
-      </c>
-      <c r="E12" s="37">
-        <v>11900000</v>
-      </c>
-      <c r="F12" s="37">
-        <v>15200000</v>
-      </c>
-      <c r="G12" s="37">
-        <v>10600000</v>
-      </c>
-      <c r="H12" s="37">
-        <v>6900000</v>
-      </c>
-      <c r="I12" s="37">
-        <v>6900000</v>
-      </c>
-      <c r="J12" s="37">
-        <v>5500000</v>
-      </c>
-      <c r="K12" s="37">
-        <v>5700000</v>
-      </c>
-      <c r="L12" s="37">
-        <f t="shared" si="36"/>
-        <v>5600000</v>
-      </c>
-      <c r="M12" s="37">
-        <f t="shared" si="37"/>
-        <v>5650000</v>
-      </c>
-      <c r="N12" s="37">
-        <f t="shared" si="38"/>
-        <v>5625000</v>
-      </c>
-      <c r="O12" s="37">
-        <f t="shared" si="39"/>
-        <v>5637500</v>
-      </c>
-      <c r="P12" s="37">
-        <f t="shared" si="40"/>
-        <v>5631250</v>
-      </c>
-      <c r="Q12" s="37">
-        <f t="shared" si="1"/>
-        <v>5634375</v>
-      </c>
-      <c r="R12" s="37">
-        <f t="shared" si="2"/>
-        <v>5632812.5</v>
-      </c>
-      <c r="S12" s="37">
-        <f t="shared" si="3"/>
-        <v>5633593.75</v>
-      </c>
-      <c r="T12" s="37">
-        <f t="shared" si="4"/>
-        <v>5633203.125</v>
-      </c>
-      <c r="U12" s="37">
-        <f t="shared" si="5"/>
-        <v>5633398.4375</v>
-      </c>
-      <c r="V12" s="37">
-        <f t="shared" si="6"/>
-        <v>5633300.78125</v>
-      </c>
-      <c r="W12" s="37">
-        <f t="shared" si="7"/>
-        <v>5633349.609375</v>
-      </c>
-      <c r="X12" s="37">
-        <f t="shared" si="8"/>
-        <v>5633325.1953125</v>
-      </c>
-      <c r="Y12" s="37">
-        <f t="shared" si="9"/>
-        <v>5633337.40234375</v>
-      </c>
-      <c r="Z12" s="37">
-        <f t="shared" si="10"/>
-        <v>5633331.298828125</v>
-      </c>
-      <c r="AA12" s="37">
-        <f t="shared" si="11"/>
-        <v>5633334.3505859375</v>
-      </c>
-      <c r="AB12" s="37">
-        <f t="shared" si="12"/>
-        <v>5633332.8247070313</v>
-      </c>
-      <c r="AC12" s="37">
-        <f t="shared" si="13"/>
-        <v>5633333.5876464844</v>
-      </c>
-      <c r="AD12" s="37">
-        <f t="shared" si="14"/>
-        <v>5633333.2061767578</v>
-      </c>
-      <c r="AE12" s="37">
-        <f t="shared" si="15"/>
-        <v>5633333.3969116211</v>
-      </c>
-      <c r="AF12" s="37">
-        <f t="shared" si="16"/>
-        <v>5633333.3015441895</v>
-      </c>
-      <c r="AG12" s="37">
-        <f t="shared" si="17"/>
-        <v>5633333.3492279053</v>
-      </c>
-      <c r="AH12" s="37">
-        <f t="shared" si="18"/>
-        <v>5633333.3253860474</v>
-      </c>
-      <c r="AI12" s="37">
-        <f t="shared" si="19"/>
-        <v>5633333.3373069763</v>
-      </c>
-      <c r="AJ12" s="37">
-        <f t="shared" si="20"/>
-        <v>5633333.3313465118</v>
-      </c>
-      <c r="AK12" s="37">
-        <f t="shared" si="21"/>
-        <v>5633333.3343267441</v>
-      </c>
-      <c r="AL12" s="37">
-        <f t="shared" si="22"/>
-        <v>5633333.332836628</v>
-      </c>
-      <c r="AM12" s="37">
-        <f t="shared" si="23"/>
-        <v>5633333.333581686</v>
-      </c>
-      <c r="AN12" s="37">
-        <f t="shared" si="24"/>
-        <v>5633333.333209157</v>
-      </c>
-      <c r="AO12" s="37">
-        <f t="shared" si="25"/>
-        <v>5633333.3333954215</v>
-      </c>
-      <c r="AP12" s="37">
-        <f t="shared" si="26"/>
-        <v>5633333.3333022892</v>
-      </c>
-      <c r="AQ12" s="37">
-        <f t="shared" si="27"/>
-        <v>5633333.3333488554</v>
-      </c>
-      <c r="AR12" s="37">
-        <f t="shared" si="28"/>
-        <v>5633333.3333255723</v>
-      </c>
-      <c r="AS12" s="37">
-        <f t="shared" si="29"/>
-        <v>5633333.3333372138</v>
-      </c>
-      <c r="AT12" s="37">
-        <f t="shared" si="30"/>
-        <v>5633333.3333313931</v>
-      </c>
-      <c r="AU12" s="37">
-        <f t="shared" si="31"/>
-        <v>5633333.3333343035</v>
-      </c>
-      <c r="AV12" s="37">
-        <f t="shared" si="32"/>
-        <v>5633333.3333328478</v>
-      </c>
-      <c r="AW12" s="37">
-        <f t="shared" si="33"/>
-        <v>5633333.3333335761</v>
-      </c>
-      <c r="AX12" s="37">
-        <f t="shared" si="34"/>
-        <v>5633333.333333212</v>
-      </c>
-      <c r="AY12" s="37">
-        <f t="shared" si="35"/>
-        <v>5633333.3333333936</v>
-      </c>
-    </row>
-    <row r="13" spans="1:51" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+      <c r="B14" s="25">
+        <v>1030200000</v>
+      </c>
+      <c r="C14" s="25">
+        <v>1268200000</v>
+      </c>
+      <c r="D14" s="25">
+        <v>1411000000</v>
+      </c>
+      <c r="E14" s="25">
+        <v>1382100000</v>
+      </c>
+      <c r="F14" s="25">
+        <v>1378700000</v>
+      </c>
+      <c r="G14" s="25">
+        <v>1356600000</v>
+      </c>
+      <c r="H14" s="25">
+        <v>1378700000</v>
+      </c>
+      <c r="I14" s="25">
+        <v>1358300000</v>
+      </c>
+      <c r="J14" s="25">
+        <v>1380400000</v>
+      </c>
+      <c r="K14" s="25">
+        <v>1399100000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>149</v>
       </c>
-      <c r="B13" s="37">
+      <c r="B15" s="37">
         <v>20500000</v>
       </c>
-      <c r="C13" s="37">
+      <c r="C15" s="37">
         <v>22200000</v>
       </c>
-      <c r="D13" s="37">
+      <c r="D15" s="37">
         <v>22600000</v>
       </c>
-      <c r="E13" s="37">
+      <c r="E15" s="37">
         <v>21600000</v>
       </c>
-      <c r="F13" s="37">
+      <c r="F15" s="37">
         <v>21700000</v>
       </c>
-      <c r="G13" s="37">
+      <c r="G15" s="37">
         <v>21100000</v>
       </c>
-      <c r="H13" s="37">
+      <c r="H15" s="37">
         <v>21400000</v>
       </c>
-      <c r="I13" s="37">
+      <c r="I15" s="37">
         <v>21200000</v>
       </c>
-      <c r="J13" s="37">
+      <c r="J15" s="37">
         <v>21400000</v>
       </c>
-      <c r="K13" s="37">
+      <c r="K15" s="37">
         <v>21500000</v>
       </c>
-      <c r="L13" s="37">
-        <f t="shared" si="36"/>
-        <v>21450000</v>
-      </c>
-      <c r="M13" s="37">
-        <f t="shared" si="37"/>
-        <v>21475000</v>
-      </c>
-      <c r="N13" s="37">
-        <f t="shared" si="38"/>
-        <v>21462500</v>
-      </c>
-      <c r="O13" s="37">
-        <f t="shared" si="39"/>
-        <v>21468750</v>
-      </c>
-      <c r="P13" s="37">
-        <f t="shared" si="40"/>
-        <v>21465625</v>
-      </c>
-      <c r="Q13" s="37">
-        <f t="shared" si="1"/>
-        <v>21467187.5</v>
-      </c>
-      <c r="R13" s="37">
-        <f t="shared" si="2"/>
-        <v>21466406.25</v>
-      </c>
-      <c r="S13" s="37">
-        <f t="shared" si="3"/>
-        <v>21466796.875</v>
-      </c>
-      <c r="T13" s="37">
-        <f t="shared" si="4"/>
-        <v>21466601.5625</v>
-      </c>
-      <c r="U13" s="37">
-        <f t="shared" si="5"/>
-        <v>21466699.21875</v>
-      </c>
-      <c r="V13" s="37">
-        <f t="shared" si="6"/>
-        <v>21466650.390625</v>
-      </c>
-      <c r="W13" s="37">
-        <f t="shared" si="7"/>
-        <v>21466674.8046875</v>
-      </c>
-      <c r="X13" s="37">
-        <f t="shared" si="8"/>
-        <v>21466662.59765625</v>
-      </c>
-      <c r="Y13" s="37">
-        <f t="shared" si="9"/>
-        <v>21466668.701171875</v>
-      </c>
-      <c r="Z13" s="37">
-        <f t="shared" si="10"/>
-        <v>21466665.649414063</v>
-      </c>
-      <c r="AA13" s="37">
-        <f t="shared" si="11"/>
-        <v>21466667.175292969</v>
-      </c>
-      <c r="AB13" s="37">
-        <f t="shared" si="12"/>
-        <v>21466666.412353516</v>
-      </c>
-      <c r="AC13" s="37">
-        <f t="shared" si="13"/>
-        <v>21466666.793823242</v>
-      </c>
-      <c r="AD13" s="37">
-        <f t="shared" si="14"/>
-        <v>21466666.603088379</v>
-      </c>
-      <c r="AE13" s="37">
-        <f t="shared" si="15"/>
-        <v>21466666.698455811</v>
-      </c>
-      <c r="AF13" s="37">
-        <f t="shared" si="16"/>
-        <v>21466666.650772095</v>
-      </c>
-      <c r="AG13" s="37">
-        <f t="shared" si="17"/>
-        <v>21466666.674613953</v>
-      </c>
-      <c r="AH13" s="37">
-        <f t="shared" si="18"/>
-        <v>21466666.662693024</v>
-      </c>
-      <c r="AI13" s="37">
-        <f t="shared" si="19"/>
-        <v>21466666.668653488</v>
-      </c>
-      <c r="AJ13" s="37">
-        <f t="shared" si="20"/>
-        <v>21466666.665673256</v>
-      </c>
-      <c r="AK13" s="37">
-        <f t="shared" si="21"/>
-        <v>21466666.667163372</v>
-      </c>
-      <c r="AL13" s="37">
-        <f t="shared" si="22"/>
-        <v>21466666.666418314</v>
-      </c>
-      <c r="AM13" s="37">
-        <f t="shared" si="23"/>
-        <v>21466666.666790843</v>
-      </c>
-      <c r="AN13" s="37">
-        <f t="shared" si="24"/>
-        <v>21466666.666604578</v>
-      </c>
-      <c r="AO13" s="37">
-        <f t="shared" si="25"/>
-        <v>21466666.666697711</v>
-      </c>
-      <c r="AP13" s="37">
-        <f t="shared" si="26"/>
-        <v>21466666.666651145</v>
-      </c>
-      <c r="AQ13" s="37">
-        <f t="shared" si="27"/>
-        <v>21466666.666674428</v>
-      </c>
-      <c r="AR13" s="37">
-        <f t="shared" si="28"/>
-        <v>21466666.666662786</v>
-      </c>
-      <c r="AS13" s="37">
-        <f t="shared" si="29"/>
-        <v>21466666.666668609</v>
-      </c>
-      <c r="AT13" s="37">
-        <f t="shared" si="30"/>
-        <v>21466666.666665696</v>
-      </c>
-      <c r="AU13" s="37">
-        <f t="shared" si="31"/>
-        <v>21466666.666667152</v>
-      </c>
-      <c r="AV13" s="37">
-        <f t="shared" si="32"/>
-        <v>21466666.666666426</v>
-      </c>
-      <c r="AW13" s="37">
-        <f t="shared" si="33"/>
-        <v>21466666.666666791</v>
-      </c>
-      <c r="AX13" s="37">
-        <f t="shared" si="34"/>
-        <v>21466666.666666608</v>
-      </c>
-      <c r="AY13" s="37">
-        <f t="shared" si="35"/>
-        <v>21466666.666666701</v>
-      </c>
-    </row>
-    <row r="14" spans="1:51" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>156</v>
       </c>
-      <c r="B14" s="37">
-        <v>5800000</v>
-      </c>
-      <c r="C14" s="37">
-        <v>6700000</v>
-      </c>
-      <c r="D14" s="37">
-        <v>7500000</v>
-      </c>
-      <c r="E14" s="37">
-        <v>7400000</v>
-      </c>
-      <c r="F14" s="37">
-        <v>7900000</v>
-      </c>
-      <c r="G14" s="37">
-        <v>7900000</v>
-      </c>
-      <c r="H14" s="37">
-        <v>8000000</v>
-      </c>
-      <c r="I14" s="37">
-        <v>7800000</v>
-      </c>
-      <c r="J14" s="37">
-        <v>7800000</v>
-      </c>
-      <c r="K14" s="37">
-        <v>7900000</v>
-      </c>
-      <c r="L14" s="37">
-        <f t="shared" si="36"/>
-        <v>7850000</v>
-      </c>
-      <c r="M14" s="37">
-        <f t="shared" si="37"/>
-        <v>7875000</v>
-      </c>
-      <c r="N14" s="37">
-        <f t="shared" si="38"/>
-        <v>7862500</v>
-      </c>
-      <c r="O14" s="37">
-        <f t="shared" si="39"/>
-        <v>7868750</v>
-      </c>
-      <c r="P14" s="37">
-        <f t="shared" si="40"/>
-        <v>7865625</v>
-      </c>
-      <c r="Q14" s="37">
-        <f t="shared" si="1"/>
-        <v>7867187.5</v>
-      </c>
-      <c r="R14" s="37">
-        <f t="shared" si="2"/>
-        <v>7866406.25</v>
-      </c>
-      <c r="S14" s="37">
-        <f t="shared" si="3"/>
-        <v>7866796.875</v>
-      </c>
-      <c r="T14" s="37">
-        <f t="shared" si="4"/>
-        <v>7866601.5625</v>
-      </c>
-      <c r="U14" s="37">
-        <f t="shared" si="5"/>
-        <v>7866699.21875</v>
-      </c>
-      <c r="V14" s="37">
-        <f t="shared" si="6"/>
-        <v>7866650.390625</v>
-      </c>
-      <c r="W14" s="37">
-        <f t="shared" si="7"/>
-        <v>7866674.8046875</v>
-      </c>
-      <c r="X14" s="37">
-        <f t="shared" si="8"/>
-        <v>7866662.59765625</v>
-      </c>
-      <c r="Y14" s="37">
-        <f t="shared" si="9"/>
-        <v>7866668.701171875</v>
-      </c>
-      <c r="Z14" s="37">
-        <f t="shared" si="10"/>
-        <v>7866665.6494140625</v>
-      </c>
-      <c r="AA14" s="37">
-        <f t="shared" si="11"/>
-        <v>7866667.1752929688</v>
-      </c>
-      <c r="AB14" s="37">
-        <f t="shared" si="12"/>
-        <v>7866666.4123535156</v>
-      </c>
-      <c r="AC14" s="37">
-        <f t="shared" si="13"/>
-        <v>7866666.7938232422</v>
-      </c>
-      <c r="AD14" s="37">
-        <f t="shared" si="14"/>
-        <v>7866666.6030883789</v>
-      </c>
-      <c r="AE14" s="37">
-        <f t="shared" si="15"/>
-        <v>7866666.6984558105</v>
-      </c>
-      <c r="AF14" s="37">
-        <f t="shared" si="16"/>
-        <v>7866666.6507720947</v>
-      </c>
-      <c r="AG14" s="37">
-        <f t="shared" si="17"/>
-        <v>7866666.6746139526</v>
-      </c>
-      <c r="AH14" s="37">
-        <f t="shared" si="18"/>
-        <v>7866666.6626930237</v>
-      </c>
-      <c r="AI14" s="37">
-        <f t="shared" si="19"/>
-        <v>7866666.6686534882</v>
-      </c>
-      <c r="AJ14" s="37">
-        <f t="shared" si="20"/>
-        <v>7866666.6656732559</v>
-      </c>
-      <c r="AK14" s="37">
-        <f t="shared" si="21"/>
-        <v>7866666.667163372</v>
-      </c>
-      <c r="AL14" s="37">
-        <f t="shared" si="22"/>
-        <v>7866666.666418314</v>
-      </c>
-      <c r="AM14" s="37">
-        <f t="shared" si="23"/>
-        <v>7866666.666790843</v>
-      </c>
-      <c r="AN14" s="37">
-        <f t="shared" si="24"/>
-        <v>7866666.6666045785</v>
-      </c>
-      <c r="AO14" s="37">
-        <f t="shared" si="25"/>
-        <v>7866666.6666977108</v>
-      </c>
-      <c r="AP14" s="37">
-        <f t="shared" si="26"/>
-        <v>7866666.6666511446</v>
-      </c>
-      <c r="AQ14" s="37">
-        <f t="shared" si="27"/>
-        <v>7866666.6666744277</v>
-      </c>
-      <c r="AR14" s="37">
-        <f t="shared" si="28"/>
-        <v>7866666.6666627862</v>
-      </c>
-      <c r="AS14" s="37">
-        <f t="shared" si="29"/>
-        <v>7866666.6666686069</v>
-      </c>
-      <c r="AT14" s="37">
-        <f t="shared" si="30"/>
-        <v>7866666.6666656965</v>
-      </c>
-      <c r="AU14" s="37">
-        <f t="shared" si="31"/>
-        <v>7866666.6666671522</v>
-      </c>
-      <c r="AV14" s="37">
-        <f t="shared" si="32"/>
-        <v>7866666.6666664239</v>
-      </c>
-      <c r="AW14" s="37">
-        <f t="shared" si="33"/>
-        <v>7866666.666666788</v>
-      </c>
-      <c r="AX14" s="37">
-        <f t="shared" si="34"/>
-        <v>7866666.6666666064</v>
-      </c>
-      <c r="AY14" s="37">
-        <f t="shared" si="35"/>
-        <v>7866666.6666666977</v>
-      </c>
-    </row>
-    <row r="15" spans="1:51" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>150</v>
-      </c>
-      <c r="B15" s="37">
-        <v>116600000</v>
-      </c>
-      <c r="C15" s="37">
-        <v>129900000</v>
-      </c>
-      <c r="D15" s="37">
-        <v>128200000</v>
-      </c>
-      <c r="E15" s="37">
-        <v>123000000</v>
-      </c>
-      <c r="F15" s="37">
-        <v>123100000</v>
-      </c>
-      <c r="G15" s="37">
-        <v>120400000</v>
-      </c>
-      <c r="H15" s="37">
-        <v>121900000</v>
-      </c>
-      <c r="I15" s="37">
-        <v>121000000</v>
-      </c>
-      <c r="J15" s="37">
-        <v>122400000</v>
-      </c>
-      <c r="K15" s="37">
-        <v>123300000</v>
-      </c>
-      <c r="L15" s="37">
-        <f t="shared" si="36"/>
-        <v>122850000</v>
-      </c>
-      <c r="M15" s="37">
-        <f t="shared" si="37"/>
-        <v>123075000</v>
-      </c>
-      <c r="N15" s="37">
-        <f t="shared" si="38"/>
-        <v>122962500</v>
-      </c>
-      <c r="O15" s="37">
-        <f t="shared" si="39"/>
-        <v>123018750</v>
-      </c>
-      <c r="P15" s="37">
-        <f t="shared" si="40"/>
-        <v>122990625</v>
-      </c>
-      <c r="Q15" s="37">
-        <f t="shared" si="1"/>
-        <v>123004687.5</v>
-      </c>
-      <c r="R15" s="37">
-        <f t="shared" si="2"/>
-        <v>122997656.25</v>
-      </c>
-      <c r="S15" s="37">
-        <f t="shared" si="3"/>
-        <v>123001171.875</v>
-      </c>
-      <c r="T15" s="37">
-        <f t="shared" si="4"/>
-        <v>122999414.0625</v>
-      </c>
-      <c r="U15" s="37">
-        <f t="shared" si="5"/>
-        <v>123000292.96875</v>
-      </c>
-      <c r="V15" s="37">
-        <f t="shared" si="6"/>
-        <v>122999853.515625</v>
-      </c>
-      <c r="W15" s="37">
-        <f t="shared" si="7"/>
-        <v>123000073.2421875</v>
-      </c>
-      <c r="X15" s="37">
-        <f t="shared" si="8"/>
-        <v>122999963.37890625</v>
-      </c>
-      <c r="Y15" s="37">
-        <f t="shared" si="9"/>
-        <v>123000018.31054688</v>
-      </c>
-      <c r="Z15" s="37">
-        <f t="shared" si="10"/>
-        <v>122999990.84472656</v>
-      </c>
-      <c r="AA15" s="37">
-        <f t="shared" si="11"/>
-        <v>123000004.57763672</v>
-      </c>
-      <c r="AB15" s="37">
-        <f t="shared" si="12"/>
-        <v>122999997.71118164</v>
-      </c>
-      <c r="AC15" s="37">
-        <f t="shared" si="13"/>
-        <v>123000001.14440918</v>
-      </c>
-      <c r="AD15" s="37">
-        <f t="shared" si="14"/>
-        <v>122999999.42779541</v>
-      </c>
-      <c r="AE15" s="37">
-        <f t="shared" si="15"/>
-        <v>123000000.28610229</v>
-      </c>
-      <c r="AF15" s="37">
-        <f t="shared" si="16"/>
-        <v>122999999.85694885</v>
-      </c>
-      <c r="AG15" s="37">
-        <f t="shared" si="17"/>
-        <v>123000000.07152557</v>
-      </c>
-      <c r="AH15" s="37">
-        <f t="shared" si="18"/>
-        <v>122999999.96423721</v>
-      </c>
-      <c r="AI15" s="37">
-        <f t="shared" si="19"/>
-        <v>123000000.01788139</v>
-      </c>
-      <c r="AJ15" s="37">
-        <f t="shared" si="20"/>
-        <v>122999999.9910593</v>
-      </c>
-      <c r="AK15" s="37">
-        <f t="shared" si="21"/>
-        <v>123000000.00447035</v>
-      </c>
-      <c r="AL15" s="37">
-        <f t="shared" si="22"/>
-        <v>122999999.99776483</v>
-      </c>
-      <c r="AM15" s="37">
-        <f t="shared" si="23"/>
-        <v>123000000.00111759</v>
-      </c>
-      <c r="AN15" s="37">
-        <f t="shared" si="24"/>
-        <v>122999999.99944121</v>
-      </c>
-      <c r="AO15" s="37">
-        <f t="shared" si="25"/>
-        <v>123000000.0002794</v>
-      </c>
-      <c r="AP15" s="37">
-        <f t="shared" si="26"/>
-        <v>122999999.9998603</v>
-      </c>
-      <c r="AQ15" s="37">
-        <f t="shared" si="27"/>
-        <v>123000000.00006986</v>
-      </c>
-      <c r="AR15" s="37">
-        <f t="shared" si="28"/>
-        <v>122999999.99996507</v>
-      </c>
-      <c r="AS15" s="37">
-        <f t="shared" si="29"/>
-        <v>123000000.00001746</v>
-      </c>
-      <c r="AT15" s="37">
-        <f t="shared" si="30"/>
-        <v>122999999.99999127</v>
-      </c>
-      <c r="AU15" s="37">
-        <f t="shared" si="31"/>
-        <v>123000000.00000437</v>
-      </c>
-      <c r="AV15" s="37">
-        <f t="shared" si="32"/>
-        <v>122999999.99999782</v>
-      </c>
-      <c r="AW15" s="37">
-        <f t="shared" si="33"/>
-        <v>123000000.0000011</v>
-      </c>
-      <c r="AX15" s="37">
-        <f t="shared" si="34"/>
-        <v>122999999.99999946</v>
-      </c>
-      <c r="AY15" s="37">
-        <f t="shared" si="35"/>
-        <v>123000000.00000028</v>
-      </c>
-    </row>
-    <row r="16" spans="1:51" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+      <c r="B16" s="37">
+        <v>58000000</v>
+      </c>
+      <c r="C16" s="37">
+        <v>67000000</v>
+      </c>
+      <c r="D16" s="37">
+        <v>75000000</v>
+      </c>
+      <c r="E16" s="37">
+        <v>74000000</v>
+      </c>
+      <c r="F16" s="37">
+        <v>79000000</v>
+      </c>
+      <c r="G16" s="37">
+        <v>79000000</v>
+      </c>
+      <c r="H16" s="37">
+        <v>80000000</v>
+      </c>
+      <c r="I16" s="37">
+        <v>78000000</v>
+      </c>
+      <c r="J16" s="37">
+        <v>78000000</v>
+      </c>
+      <c r="K16" s="37">
+        <v>79000000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>151</v>
       </c>
-      <c r="B16" s="37">
-        <v>104600000</v>
-      </c>
-      <c r="C16" s="37">
-        <v>122100000</v>
-      </c>
-      <c r="D16" s="37">
-        <v>131700000</v>
-      </c>
-      <c r="E16" s="37">
-        <v>128600000</v>
-      </c>
-      <c r="F16" s="37">
-        <v>128700000</v>
-      </c>
-      <c r="G16" s="37">
-        <v>125200000</v>
-      </c>
-      <c r="H16" s="37">
-        <v>127600000</v>
-      </c>
-      <c r="I16" s="37">
-        <v>126000000</v>
-      </c>
-      <c r="J16" s="37">
-        <v>127400000</v>
-      </c>
-      <c r="K16" s="37">
-        <v>128200000</v>
-      </c>
-      <c r="L16" s="37">
-        <f t="shared" si="36"/>
-        <v>127800000</v>
-      </c>
-      <c r="M16" s="37">
-        <f t="shared" si="37"/>
-        <v>128000000</v>
-      </c>
-      <c r="N16" s="37">
-        <f t="shared" si="38"/>
-        <v>127900000</v>
-      </c>
-      <c r="O16" s="37">
-        <f t="shared" si="39"/>
-        <v>127950000</v>
-      </c>
-      <c r="P16" s="37">
-        <f t="shared" si="40"/>
-        <v>127925000</v>
-      </c>
-      <c r="Q16" s="37">
-        <f t="shared" si="1"/>
-        <v>127937500</v>
-      </c>
-      <c r="R16" s="37">
-        <f t="shared" si="2"/>
-        <v>127931250</v>
-      </c>
-      <c r="S16" s="37">
-        <f t="shared" si="3"/>
-        <v>127934375</v>
-      </c>
-      <c r="T16" s="37">
-        <f t="shared" si="4"/>
-        <v>127932812.5</v>
-      </c>
-      <c r="U16" s="37">
-        <f t="shared" si="5"/>
-        <v>127933593.75</v>
-      </c>
-      <c r="V16" s="37">
-        <f t="shared" si="6"/>
-        <v>127933203.125</v>
-      </c>
-      <c r="W16" s="37">
-        <f t="shared" si="7"/>
-        <v>127933398.4375</v>
-      </c>
-      <c r="X16" s="37">
-        <f t="shared" si="8"/>
-        <v>127933300.78125</v>
-      </c>
-      <c r="Y16" s="37">
-        <f t="shared" si="9"/>
-        <v>127933349.609375</v>
-      </c>
-      <c r="Z16" s="37">
-        <f t="shared" si="10"/>
-        <v>127933325.1953125</v>
-      </c>
-      <c r="AA16" s="37">
-        <f t="shared" si="11"/>
-        <v>127933337.40234375</v>
-      </c>
-      <c r="AB16" s="37">
-        <f t="shared" si="12"/>
-        <v>127933331.29882813</v>
-      </c>
-      <c r="AC16" s="37">
-        <f t="shared" si="13"/>
-        <v>127933334.35058594</v>
-      </c>
-      <c r="AD16" s="37">
-        <f t="shared" si="14"/>
-        <v>127933332.82470703</v>
-      </c>
-      <c r="AE16" s="37">
-        <f t="shared" si="15"/>
-        <v>127933333.58764648</v>
-      </c>
-      <c r="AF16" s="37">
-        <f t="shared" si="16"/>
-        <v>127933333.20617676</v>
-      </c>
-      <c r="AG16" s="37">
-        <f t="shared" si="17"/>
-        <v>127933333.39691162</v>
-      </c>
-      <c r="AH16" s="37">
-        <f t="shared" si="18"/>
-        <v>127933333.30154419</v>
-      </c>
-      <c r="AI16" s="37">
-        <f t="shared" si="19"/>
-        <v>127933333.34922791</v>
-      </c>
-      <c r="AJ16" s="37">
-        <f t="shared" si="20"/>
-        <v>127933333.32538605</v>
-      </c>
-      <c r="AK16" s="37">
-        <f t="shared" si="21"/>
-        <v>127933333.33730698</v>
-      </c>
-      <c r="AL16" s="37">
-        <f t="shared" si="22"/>
-        <v>127933333.33134651</v>
-      </c>
-      <c r="AM16" s="37">
-        <f t="shared" si="23"/>
-        <v>127933333.33432674</v>
-      </c>
-      <c r="AN16" s="37">
-        <f t="shared" si="24"/>
-        <v>127933333.33283663</v>
-      </c>
-      <c r="AO16" s="37">
-        <f t="shared" si="25"/>
-        <v>127933333.33358169</v>
-      </c>
-      <c r="AP16" s="37">
-        <f t="shared" si="26"/>
-        <v>127933333.33320916</v>
-      </c>
-      <c r="AQ16" s="37">
-        <f t="shared" si="27"/>
-        <v>127933333.33339542</v>
-      </c>
-      <c r="AR16" s="37">
-        <f t="shared" si="28"/>
-        <v>127933333.33330229</v>
-      </c>
-      <c r="AS16" s="37">
-        <f t="shared" si="29"/>
-        <v>127933333.33334886</v>
-      </c>
-      <c r="AT16" s="37">
-        <f t="shared" si="30"/>
-        <v>127933333.33332556</v>
-      </c>
-      <c r="AU16" s="37">
-        <f t="shared" si="31"/>
-        <v>127933333.33333722</v>
-      </c>
-      <c r="AV16" s="37">
-        <f t="shared" si="32"/>
-        <v>127933333.33333139</v>
-      </c>
-      <c r="AW16" s="37">
-        <f t="shared" si="33"/>
-        <v>127933333.3333343</v>
-      </c>
-      <c r="AX16" s="37">
-        <f t="shared" si="34"/>
-        <v>127933333.33333284</v>
-      </c>
-      <c r="AY16" s="37">
-        <f t="shared" si="35"/>
-        <v>127933333.33333357</v>
-      </c>
-    </row>
-    <row r="17" spans="1:51" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>152</v>
-      </c>
-      <c r="B17" s="41">
-        <v>969375250</v>
-      </c>
-      <c r="C17">
-        <v>1001504250</v>
-      </c>
-      <c r="D17">
-        <v>1046900000</v>
-      </c>
-      <c r="E17">
-        <v>1007009500</v>
-      </c>
-      <c r="F17">
-        <v>1030294000</v>
-      </c>
-      <c r="G17">
-        <v>1075328750</v>
-      </c>
-      <c r="H17">
-        <v>1011161000</v>
-      </c>
-      <c r="I17">
-        <v>1076231250</v>
-      </c>
-      <c r="J17">
-        <v>1028128000</v>
-      </c>
-      <c r="K17">
-        <v>1055564000</v>
-      </c>
-      <c r="L17" s="37">
-        <f t="shared" si="36"/>
-        <v>1041846000</v>
-      </c>
-      <c r="M17" s="37">
-        <f t="shared" si="37"/>
-        <v>1048705000</v>
-      </c>
-      <c r="N17" s="37">
-        <f t="shared" si="38"/>
-        <v>1045275500</v>
-      </c>
-      <c r="O17" s="37">
-        <f t="shared" si="39"/>
-        <v>1046990250</v>
-      </c>
-      <c r="P17" s="37">
-        <f t="shared" si="40"/>
-        <v>1046132875</v>
-      </c>
-      <c r="Q17" s="37">
-        <f t="shared" si="1"/>
-        <v>1046561562.5</v>
-      </c>
-      <c r="R17" s="37">
-        <f t="shared" si="2"/>
-        <v>1046347218.75</v>
-      </c>
-      <c r="S17" s="37">
-        <f t="shared" si="3"/>
-        <v>1046454390.625</v>
-      </c>
-      <c r="T17" s="37">
-        <f t="shared" si="4"/>
-        <v>1046400804.6875</v>
-      </c>
-      <c r="U17" s="37">
-        <f t="shared" si="5"/>
-        <v>1046427597.65625</v>
-      </c>
-      <c r="V17" s="37">
-        <f t="shared" si="6"/>
-        <v>1046414201.171875</v>
-      </c>
-      <c r="W17" s="37">
-        <f t="shared" si="7"/>
-        <v>1046420899.4140625</v>
-      </c>
-      <c r="X17" s="37">
-        <f t="shared" si="8"/>
-        <v>1046417550.2929688</v>
-      </c>
-      <c r="Y17" s="37">
-        <f t="shared" si="9"/>
-        <v>1046419224.8535156</v>
-      </c>
-      <c r="Z17" s="37">
-        <f t="shared" si="10"/>
-        <v>1046418387.5732422</v>
-      </c>
-      <c r="AA17" s="37">
-        <f t="shared" si="11"/>
-        <v>1046418806.2133789</v>
-      </c>
-      <c r="AB17" s="37">
-        <f t="shared" si="12"/>
-        <v>1046418596.8933105</v>
-      </c>
-      <c r="AC17" s="37">
-        <f t="shared" si="13"/>
-        <v>1046418701.5533447</v>
-      </c>
-      <c r="AD17" s="37">
-        <f t="shared" si="14"/>
-        <v>1046418649.2233276</v>
-      </c>
-      <c r="AE17" s="37">
-        <f t="shared" si="15"/>
-        <v>1046418675.3883362</v>
-      </c>
-      <c r="AF17" s="37">
-        <f t="shared" si="16"/>
-        <v>1046418662.3058319</v>
-      </c>
-      <c r="AG17" s="37">
-        <f t="shared" si="17"/>
-        <v>1046418668.847084</v>
-      </c>
-      <c r="AH17" s="37">
-        <f t="shared" si="18"/>
-        <v>1046418665.576458</v>
-      </c>
-      <c r="AI17" s="37">
-        <f t="shared" si="19"/>
-        <v>1046418667.211771</v>
-      </c>
-      <c r="AJ17" s="37">
-        <f t="shared" si="20"/>
-        <v>1046418666.3941145</v>
-      </c>
-      <c r="AK17" s="37">
-        <f t="shared" si="21"/>
-        <v>1046418666.8029428</v>
-      </c>
-      <c r="AL17" s="37">
-        <f t="shared" si="22"/>
-        <v>1046418666.5985286</v>
-      </c>
-      <c r="AM17" s="37">
-        <f t="shared" si="23"/>
-        <v>1046418666.7007357</v>
-      </c>
-      <c r="AN17" s="37">
-        <f t="shared" si="24"/>
-        <v>1046418666.6496322</v>
-      </c>
-      <c r="AO17" s="37">
-        <f t="shared" si="25"/>
-        <v>1046418666.675184</v>
-      </c>
-      <c r="AP17" s="37">
-        <f t="shared" si="26"/>
-        <v>1046418666.6624081</v>
-      </c>
-      <c r="AQ17" s="37">
-        <f t="shared" si="27"/>
-        <v>1046418666.6687961</v>
-      </c>
-      <c r="AR17" s="37">
-        <f t="shared" si="28"/>
-        <v>1046418666.6656021</v>
-      </c>
-      <c r="AS17" s="37">
-        <f t="shared" si="29"/>
-        <v>1046418666.6671991</v>
-      </c>
-      <c r="AT17" s="37">
-        <f t="shared" si="30"/>
-        <v>1046418666.6664007</v>
-      </c>
-      <c r="AU17" s="37">
-        <f t="shared" si="31"/>
-        <v>1046418666.6667999</v>
-      </c>
-      <c r="AV17" s="37">
-        <f t="shared" si="32"/>
-        <v>1046418666.6666002</v>
-      </c>
-      <c r="AW17" s="37">
-        <f t="shared" si="33"/>
-        <v>1046418666.6667001</v>
-      </c>
-      <c r="AX17" s="37">
-        <f t="shared" si="34"/>
-        <v>1046418666.6666502</v>
-      </c>
-      <c r="AY17" s="37">
-        <f t="shared" si="35"/>
-        <v>1046418666.6666751</v>
-      </c>
-    </row>
-    <row r="18" spans="1:51" x14ac:dyDescent="0.25">
+      <c r="B17" s="37">
+        <v>1046000000</v>
+      </c>
+      <c r="C17" s="37">
+        <v>1221000000</v>
+      </c>
+      <c r="D17" s="37">
+        <v>1317000000</v>
+      </c>
+      <c r="E17" s="37">
+        <v>1286000000</v>
+      </c>
+      <c r="F17" s="37">
+        <v>1287000000</v>
+      </c>
+      <c r="G17" s="37">
+        <v>1252000000</v>
+      </c>
+      <c r="H17" s="37">
+        <v>1276000000</v>
+      </c>
+      <c r="I17" s="37">
+        <v>1260000000</v>
+      </c>
+      <c r="J17" s="37">
+        <v>1274000000</v>
+      </c>
+      <c r="K17" s="37">
+        <v>1282000000</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>153</v>
       </c>
       <c r="B18" s="25">
-        <v>500000</v>
+        <v>50000000</v>
       </c>
       <c r="C18" s="25">
-        <v>500000</v>
+        <v>50000000</v>
       </c>
       <c r="D18" s="25">
-        <v>700000</v>
+        <v>70000000</v>
       </c>
       <c r="E18" s="25">
-        <v>2000000</v>
+        <v>200000000</v>
       </c>
       <c r="F18" s="25">
-        <v>2500000</v>
+        <v>250000000</v>
       </c>
       <c r="G18" s="25">
-        <v>1800000</v>
+        <v>180000000</v>
       </c>
       <c r="H18" s="25">
-        <v>1200000</v>
+        <v>120000000</v>
       </c>
       <c r="I18" s="25">
-        <v>1200000</v>
+        <v>120000000</v>
       </c>
       <c r="J18" s="25">
-        <v>900000</v>
+        <v>90000000</v>
       </c>
       <c r="K18" s="25">
-        <v>1000000</v>
-      </c>
-      <c r="L18" s="37">
-        <f>AVERAGE(I18:K18)</f>
-        <v>1033333.3333333334</v>
-      </c>
-      <c r="M18" s="37">
-        <f t="shared" si="37"/>
-        <v>1016666.6666666667</v>
-      </c>
-      <c r="N18" s="37">
-        <f t="shared" si="38"/>
-        <v>1025000</v>
-      </c>
-      <c r="O18" s="37">
-        <f t="shared" si="39"/>
-        <v>1020833.3333333334</v>
-      </c>
-      <c r="P18" s="37">
-        <f t="shared" si="40"/>
-        <v>1022916.6666666667</v>
-      </c>
-      <c r="Q18" s="37">
-        <f t="shared" si="1"/>
-        <v>1021875</v>
-      </c>
-      <c r="R18" s="37">
-        <f t="shared" si="2"/>
-        <v>1022395.8333333334</v>
-      </c>
-      <c r="S18" s="37">
-        <f t="shared" si="3"/>
-        <v>1022135.4166666667</v>
-      </c>
-      <c r="T18" s="37">
-        <f t="shared" si="4"/>
-        <v>1022265.625</v>
-      </c>
-      <c r="U18" s="37">
-        <f t="shared" si="5"/>
-        <v>1022200.5208333334</v>
-      </c>
-      <c r="V18" s="37">
-        <f t="shared" si="6"/>
-        <v>1022233.0729166667</v>
-      </c>
-      <c r="W18" s="37">
-        <f t="shared" si="7"/>
-        <v>1022216.796875</v>
-      </c>
-      <c r="X18" s="37">
-        <f t="shared" si="8"/>
-        <v>1022224.9348958334</v>
-      </c>
-      <c r="Y18" s="37">
-        <f t="shared" si="9"/>
-        <v>1022220.8658854167</v>
-      </c>
-      <c r="Z18" s="37">
-        <f t="shared" si="10"/>
-        <v>1022222.900390625</v>
-      </c>
-      <c r="AA18" s="37">
-        <f t="shared" si="11"/>
-        <v>1022221.8831380209</v>
-      </c>
-      <c r="AB18" s="37">
-        <f t="shared" si="12"/>
-        <v>1022222.391764323</v>
-      </c>
-      <c r="AC18" s="37">
-        <f t="shared" si="13"/>
-        <v>1022222.1374511719</v>
-      </c>
-      <c r="AD18" s="37">
-        <f t="shared" si="14"/>
-        <v>1022222.2646077474</v>
-      </c>
-      <c r="AE18" s="37">
-        <f t="shared" si="15"/>
-        <v>1022222.2010294597</v>
-      </c>
-      <c r="AF18" s="37">
-        <f t="shared" si="16"/>
-        <v>1022222.2328186035</v>
-      </c>
-      <c r="AG18" s="37">
-        <f t="shared" si="17"/>
-        <v>1022222.2169240316</v>
-      </c>
-      <c r="AH18" s="37">
-        <f t="shared" si="18"/>
-        <v>1022222.2248713176</v>
-      </c>
-      <c r="AI18" s="37">
-        <f t="shared" si="19"/>
-        <v>1022222.2208976746</v>
-      </c>
-      <c r="AJ18" s="37">
-        <f t="shared" si="20"/>
-        <v>1022222.2228844961</v>
-      </c>
-      <c r="AK18" s="37">
-        <f t="shared" si="21"/>
-        <v>1022222.2218910854</v>
-      </c>
-      <c r="AL18" s="37">
-        <f t="shared" si="22"/>
-        <v>1022222.2223877907</v>
-      </c>
-      <c r="AM18" s="37">
-        <f t="shared" si="23"/>
-        <v>1022222.222139438</v>
-      </c>
-      <c r="AN18" s="37">
-        <f t="shared" si="24"/>
-        <v>1022222.2222636144</v>
-      </c>
-      <c r="AO18" s="37">
-        <f t="shared" si="25"/>
-        <v>1022222.2222015262</v>
-      </c>
-      <c r="AP18" s="37">
-        <f t="shared" si="26"/>
-        <v>1022222.2222325703</v>
-      </c>
-      <c r="AQ18" s="37">
-        <f t="shared" si="27"/>
-        <v>1022222.2222170483</v>
-      </c>
-      <c r="AR18" s="37">
-        <f t="shared" si="28"/>
-        <v>1022222.2222248092</v>
-      </c>
-      <c r="AS18" s="37">
-        <f t="shared" si="29"/>
-        <v>1022222.2222209288</v>
-      </c>
-      <c r="AT18" s="37">
-        <f t="shared" si="30"/>
-        <v>1022222.2222228691</v>
-      </c>
-      <c r="AU18" s="37">
-        <f t="shared" si="31"/>
-        <v>1022222.2222218988</v>
-      </c>
-      <c r="AV18" s="37">
-        <f t="shared" si="32"/>
-        <v>1022222.2222223839</v>
-      </c>
-      <c r="AW18" s="37">
-        <f t="shared" si="33"/>
-        <v>1022222.2222221415</v>
-      </c>
-      <c r="AX18" s="37">
-        <f t="shared" si="34"/>
-        <v>1022222.2222222628</v>
-      </c>
-      <c r="AY18" s="37">
-        <f t="shared" si="35"/>
-        <v>1022222.2222222021</v>
-      </c>
-    </row>
-    <row r="19" spans="1:51" x14ac:dyDescent="0.25">
+        <v>100000000</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B19" s="25"/>
       <c r="C19" s="25"/>
       <c r="D19" s="25"/>
@@ -22070,42 +19221,46 @@
       <c r="H19" s="25"/>
       <c r="I19" s="25"/>
       <c r="J19" s="25"/>
-    </row>
-    <row r="20" spans="1:51" x14ac:dyDescent="0.25">
-      <c r="B20" s="42"/>
-      <c r="C20" s="42"/>
-      <c r="D20" s="42"/>
-      <c r="E20" s="42"/>
-      <c r="F20" s="42"/>
-      <c r="G20" s="42"/>
-      <c r="H20" s="42"/>
-      <c r="I20" s="42"/>
-      <c r="J20" s="42"/>
-    </row>
-    <row r="21" spans="1:51" x14ac:dyDescent="0.25">
-      <c r="B21" s="41"/>
-      <c r="C21" s="41"/>
-      <c r="D21" s="25"/>
-      <c r="E21" s="25"/>
-      <c r="F21" s="25"/>
-      <c r="G21" s="25"/>
-      <c r="H21" s="25"/>
-      <c r="I21" s="25"/>
-      <c r="J21" s="25"/>
-    </row>
-    <row r="22" spans="1:51" x14ac:dyDescent="0.25">
+      <c r="K19" s="25"/>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B20" s="37"/>
+      <c r="C20" s="37"/>
+      <c r="D20" s="37"/>
+      <c r="E20" s="37"/>
+      <c r="F20" s="37"/>
+      <c r="G20" s="37"/>
+      <c r="H20" s="37"/>
+      <c r="I20" s="37"/>
+      <c r="J20" s="37"/>
+      <c r="K20" s="37"/>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B21" s="42"/>
+      <c r="C21" s="42"/>
+      <c r="D21" s="42"/>
+      <c r="E21" s="42"/>
+      <c r="F21" s="42"/>
+      <c r="G21" s="42"/>
+      <c r="H21" s="42"/>
+      <c r="I21" s="42"/>
+      <c r="J21" s="42"/>
+      <c r="K21" s="42"/>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B22" s="41"/>
-      <c r="C22" s="41"/>
-      <c r="D22" s="25"/>
-      <c r="E22" s="25"/>
-      <c r="F22" s="25"/>
-      <c r="G22" s="25"/>
-      <c r="H22" s="25"/>
-      <c r="I22" s="25"/>
-      <c r="J22" s="25"/>
-    </row>
-    <row r="23" spans="1:51" x14ac:dyDescent="0.25">
-      <c r="B23" s="25"/>
+      <c r="C22" s="42"/>
+      <c r="D22" s="42"/>
+      <c r="E22" s="42"/>
+      <c r="F22" s="42"/>
+      <c r="G22" s="42"/>
+      <c r="H22" s="42"/>
+      <c r="I22" s="42"/>
+      <c r="J22" s="42"/>
+      <c r="K22" s="42"/>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B23" s="37"/>
       <c r="C23" s="25"/>
       <c r="D23" s="25"/>
       <c r="E23" s="40"/>
@@ -22116,7 +19271,7 @@
       <c r="J23" s="25"/>
       <c r="K23" s="25"/>
     </row>
-    <row r="24" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B24" s="25"/>
       <c r="C24" s="25"/>
       <c r="D24" s="25"/>
@@ -22128,7 +19283,7 @@
       <c r="J24" s="25"/>
       <c r="K24" s="25"/>
     </row>
-    <row r="25" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B25" s="25"/>
       <c r="C25" s="25"/>
       <c r="D25" s="25"/>
@@ -22140,7 +19295,7 @@
       <c r="J25" s="25"/>
       <c r="K25" s="25"/>
     </row>
-    <row r="26" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B26" s="25"/>
       <c r="C26" s="25"/>
       <c r="D26" s="25"/>
@@ -22152,7 +19307,7 @@
       <c r="J26" s="25"/>
       <c r="K26" s="25"/>
     </row>
-    <row r="27" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B27" s="25"/>
       <c r="C27" s="25"/>
       <c r="D27" s="25"/>
@@ -22164,7 +19319,7 @@
       <c r="J27" s="25"/>
       <c r="K27" s="25"/>
     </row>
-    <row r="28" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B28" s="25"/>
       <c r="C28" s="25"/>
       <c r="D28" s="25"/>
@@ -22176,7 +19331,7 @@
       <c r="J28" s="25"/>
       <c r="K28" s="25"/>
     </row>
-    <row r="29" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B29" s="25"/>
       <c r="C29" s="25"/>
       <c r="D29" s="25"/>
@@ -22188,7 +19343,7 @@
       <c r="J29" s="25"/>
       <c r="K29" s="25"/>
     </row>
-    <row r="30" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B30" s="25"/>
       <c r="C30" s="25"/>
       <c r="D30" s="25"/>
@@ -22200,7 +19355,7 @@
       <c r="J30" s="25"/>
       <c r="K30" s="25"/>
     </row>
-    <row r="31" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B31" s="25"/>
       <c r="C31" s="25"/>
       <c r="D31" s="25"/>
@@ -22212,7 +19367,7 @@
       <c r="J31" s="25"/>
       <c r="K31" s="25"/>
     </row>
-    <row r="32" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B32" s="25"/>
       <c r="C32" s="25"/>
       <c r="D32" s="25"/>
@@ -22369,16 +19524,11 @@
       <c r="K44" s="25"/>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="4294967293" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7AEDCBEC-A12F-4CB4-BD24-1D1201B71C25}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <autoFilter ref="A1:K18" xr:uid="{8DF17EB8-02F1-485E-9D81-51CF2F0BE0EA}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K18">
+      <sortCondition ref="A1:A18"/>
+    </sortState>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>